<commit_message>
Actualización automática 2026-09-17 11:30:18
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -837,7 +837,7 @@
         <v>0</v>
       </c>
       <c r="M6" s="2" t="n">
-        <v>0</v>
+        <v>708.88</v>
       </c>
       <c r="N6" s="2" t="n">
         <v>0</v>
@@ -2037,7 +2037,7 @@
         <v>0</v>
       </c>
       <c r="M26" s="2" t="n">
-        <v>0</v>
+        <v>5779.47</v>
       </c>
       <c r="N26" s="2" t="n">
         <v>0</v>
@@ -4028,7 +4028,7 @@
       </c>
       <c r="M59" s="3" t="inlineStr">
         <is>
-          <t>7 de 57</t>
+          <t>9 de 57</t>
         </is>
       </c>
       <c r="N59" s="3" t="inlineStr">
@@ -4300,7 +4300,7 @@
         <v>0</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>0</v>
+        <v>708.88</v>
       </c>
       <c r="G8" s="2" t="n">
         <v>1000</v>
@@ -4732,7 +4732,7 @@
         <v>11932.7</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>1830.72</v>
+        <v>7610.19</v>
       </c>
       <c r="G24" s="2" t="n">
         <v>4000</v>
@@ -5505,7 +5505,7 @@
         <v>43533.43</v>
       </c>
       <c r="F53" s="4" t="n">
-        <v>23554.01</v>
+        <v>30042.36</v>
       </c>
       <c r="G53" s="4" t="n">
         <v>47200</v>
@@ -5820,13 +5820,13 @@
         <v>39603</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>14534.82</v>
+        <v>21023.17</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>25068.18</v>
+        <v>18579.83</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0.3670131050677979</v>
+        <v>0.5308479155619523</v>
       </c>
     </row>
     <row r="13">
@@ -5839,13 +5839,13 @@
         <v>49040.76</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>23619.8</v>
+        <v>30108.15</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>25420.96</v>
+        <v>18932.61</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>0.4816360920997146</v>
+        <v>0.6139413418552241</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-22 14:30:18
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R59"/>
+  <dimension ref="A1:R60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -623,7 +623,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ALTAMIRANO VILLAVICENCIO JUAN ALEJANDRO</t>
+          <t>ALTAMIRANO MARCATOMA MARIA ANA</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
@@ -657,7 +657,7 @@
         <v>0</v>
       </c>
       <c r="M3" s="2" t="n">
-        <v>0</v>
+        <v>1328.44</v>
       </c>
       <c r="N3" s="2" t="n">
         <v>0</v>
@@ -683,7 +683,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ALVAREZ SAAVEDRA EDWIN GEOVANNY</t>
+          <t>ALTAMIRANO VILLAVICENCIO JUAN ALEJANDRO</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
@@ -743,7 +743,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ARIAS CARDENAS BOLIVAR MAURICIO</t>
+          <t>ALVAREZ SAAVEDRA EDWIN GEOVANNY</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
@@ -803,7 +803,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ARMIJOS SALINAS LUIS CLAUDIO</t>
+          <t>ARIAS CARDENAS BOLIVAR MAURICIO</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
@@ -837,7 +837,7 @@
         <v>0</v>
       </c>
       <c r="M6" s="2" t="n">
-        <v>708.88</v>
+        <v>0</v>
       </c>
       <c r="N6" s="2" t="n">
         <v>0</v>
@@ -863,7 +863,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ASES GAVILANEZ FAUSTO HERNAN</t>
+          <t>ARMIJOS SALINAS LUIS CLAUDIO</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
@@ -897,7 +897,7 @@
         <v>0</v>
       </c>
       <c r="M7" s="2" t="n">
-        <v>0</v>
+        <v>708.88</v>
       </c>
       <c r="N7" s="2" t="n">
         <v>0</v>
@@ -923,7 +923,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>BARROS YUNGA DIEGO VINICIO</t>
+          <t>ASES GAVILANEZ FAUSTO HERNAN</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
@@ -942,7 +942,7 @@
         <v>0</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>620.73</v>
+        <v>0</v>
       </c>
       <c r="I8" s="2" t="n">
         <v>0</v>
@@ -983,7 +983,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>BRAVO MONTENEGRO DANIEL ANDRES</t>
+          <t>BARROS YUNGA DIEGO VINICIO</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
@@ -1002,7 +1002,7 @@
         <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>0</v>
+        <v>620.73</v>
       </c>
       <c r="I9" s="2" t="n">
         <v>0</v>
@@ -1043,7 +1043,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CARRION MORALES CARLOS ENRIQUE</t>
+          <t>BRAVO MONTENEGRO DANIEL ANDRES</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
@@ -1103,7 +1103,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>COMERCIAL LUNA PAZMIÑO CIA. LTDA.</t>
+          <t>CARRION MORALES CARLOS ENRIQUE</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
@@ -1163,7 +1163,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>COMERCIALIZADORA RAMIREZ GALVAN CIA. LTDA</t>
+          <t>COMERCIAL LUNA PAZMIÑO CIA. LTDA.</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
@@ -1223,7 +1223,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>CORONEL PINOS CLARA MARIA</t>
+          <t>COMERCIALIZADORA RAMIREZ GALVAN CIA. LTDA</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>CORPORACION AREVALO-YUMBLA E HIJOS</t>
+          <t>CORONEL PINOS CLARA MARIA</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
@@ -1302,16 +1302,16 @@
         <v>0</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>324.9</v>
+        <v>0</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>293.58</v>
+        <v>0</v>
       </c>
       <c r="J14" s="2" t="n">
         <v>0</v>
       </c>
       <c r="K14" s="2" t="n">
-        <v>213.18</v>
+        <v>0</v>
       </c>
       <c r="L14" s="2" t="n">
         <v>0</v>
@@ -1343,7 +1343,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>DIAZ CHAVEZ DIEGO FERNANDO</t>
+          <t>CORPORACION AREVALO-YUMBLA E HIJOS</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
@@ -1362,16 +1362,16 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>0</v>
+        <v>324.9</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>0</v>
+        <v>293.58</v>
       </c>
       <c r="J15" s="2" t="n">
         <v>0</v>
       </c>
       <c r="K15" s="2" t="n">
-        <v>0</v>
+        <v>213.18</v>
       </c>
       <c r="L15" s="2" t="n">
         <v>0</v>
@@ -1403,7 +1403,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>DISTRIBUIDORA VASQUEZ ORDOÑEZ DISTRIVASOR CIA LTDA</t>
+          <t>DIAZ CHAVEZ DIEGO FERNANDO</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
@@ -1463,7 +1463,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ESPINOZA GOMEZ LILIA ROSARIO</t>
+          <t>DISTRIBUIDORA VASQUEZ ORDOÑEZ DISTRIVASOR CIA LTDA</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
@@ -1523,7 +1523,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>FABIMP BENIGNO BRAVO S.A.S.</t>
+          <t>ESPINOZA GOMEZ LILIA ROSARIO</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
@@ -1557,7 +1557,7 @@
         <v>0</v>
       </c>
       <c r="M18" s="2" t="n">
-        <v>6241.39</v>
+        <v>0</v>
       </c>
       <c r="N18" s="2" t="n">
         <v>0</v>
@@ -1583,7 +1583,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>FERRICENTER EL ARENAL CIA. LTDA.</t>
+          <t>FABIMP BENIGNO BRAVO S.A.S.</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
@@ -1617,7 +1617,7 @@
         <v>0</v>
       </c>
       <c r="M19" s="2" t="n">
-        <v>0</v>
+        <v>6241.39</v>
       </c>
       <c r="N19" s="2" t="n">
         <v>0</v>
@@ -1643,7 +1643,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>FERRICRAFT S.A.S.</t>
+          <t>FERRICENTER EL ARENAL CIA. LTDA.</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
@@ -1703,7 +1703,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>FRANK FERRETERIA FRANKFERRE CIA.</t>
+          <t>FERRICRAFT S.A.S.</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
@@ -1763,7 +1763,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>GLOBAL MOYANO &amp; ASOCIADOS LEMO S.A.S.</t>
+          <t>FRANK FERRETERIA FRANKFERRE CIA.</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
@@ -1797,7 +1797,7 @@
         <v>0</v>
       </c>
       <c r="M22" s="2" t="n">
-        <v>6.32</v>
+        <v>0</v>
       </c>
       <c r="N22" s="2" t="n">
         <v>0</v>
@@ -1823,7 +1823,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>GRANDA SANDOVAL JACKELINE ELIZABETH</t>
+          <t>GLOBAL MOYANO &amp; ASOCIADOS LEMO S.A.S.</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
@@ -1857,7 +1857,7 @@
         <v>0</v>
       </c>
       <c r="M23" s="2" t="n">
-        <v>0</v>
+        <v>6.32</v>
       </c>
       <c r="N23" s="2" t="n">
         <v>0</v>
@@ -1883,7 +1883,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>HUERTA MUÑOZ NANCY ELIZABETH</t>
+          <t>GRANDA SANDOVAL JACKELINE ELIZABETH</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
@@ -1943,7 +1943,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+          <t>HUERTA MUÑOZ NANCY ELIZABETH</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
@@ -1953,7 +1953,7 @@
         <v>0</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>65.79000000000001</v>
+        <v>0</v>
       </c>
       <c r="F25" s="2" t="n">
         <v>0</v>
@@ -2003,7 +2003,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>IMPORTADORA ORTEGA CIA. LTDA.</t>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
@@ -2013,7 +2013,7 @@
         <v>0</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>0</v>
+        <v>65.79000000000001</v>
       </c>
       <c r="F26" s="2" t="n">
         <v>0</v>
@@ -2025,7 +2025,7 @@
         <v>0</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>1830.72</v>
+        <v>0</v>
       </c>
       <c r="J26" s="2" t="n">
         <v>0</v>
@@ -2037,7 +2037,7 @@
         <v>0</v>
       </c>
       <c r="M26" s="2" t="n">
-        <v>5779.47</v>
+        <v>0</v>
       </c>
       <c r="N26" s="2" t="n">
         <v>0</v>
@@ -2063,17 +2063,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>JIMBO BRITO SELENE PATRICIA</t>
+          <t>IMPORTADORA ORTEGA CIA. LTDA.</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>436.55</v>
+        <v>0</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>417.01</v>
+        <v>0</v>
       </c>
       <c r="F27" s="2" t="n">
         <v>0</v>
@@ -2082,22 +2082,22 @@
         <v>0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>247.5</v>
+        <v>0</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>350.77</v>
+        <v>1830.72</v>
       </c>
       <c r="J27" s="2" t="n">
         <v>0</v>
       </c>
       <c r="K27" s="2" t="n">
-        <v>363.16</v>
+        <v>0</v>
       </c>
       <c r="L27" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M27" s="2" t="n">
-        <v>1918.73</v>
+        <v>5779.47</v>
       </c>
       <c r="N27" s="2" t="n">
         <v>0</v>
@@ -2123,17 +2123,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>JIMENEZ GORDILLO LADY KARINA</t>
+          <t>JIMBO BRITO SELENE PATRICIA</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>0</v>
+        <v>436.55</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>0</v>
+        <v>417.01</v>
       </c>
       <c r="F28" s="2" t="n">
         <v>0</v>
@@ -2142,22 +2142,22 @@
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>0</v>
+        <v>247.5</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>0</v>
+        <v>350.77</v>
       </c>
       <c r="J28" s="2" t="n">
         <v>0</v>
       </c>
       <c r="K28" s="2" t="n">
-        <v>0</v>
+        <v>363.16</v>
       </c>
       <c r="L28" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M28" s="2" t="n">
-        <v>0</v>
+        <v>1918.73</v>
       </c>
       <c r="N28" s="2" t="n">
         <v>0</v>
@@ -2183,7 +2183,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>JUAREZ FLORES JORGE WILLIAMS</t>
+          <t>JIMENEZ GORDILLO LADY KARINA</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
@@ -2243,7 +2243,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>LEMA ESPINOZA MANUEL MARIA</t>
+          <t>JUAREZ FLORES JORGE WILLIAMS</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
@@ -2303,7 +2303,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>MEGGA-FRANK SAS</t>
+          <t>LEMA ESPINOZA MANUEL MARIA</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
@@ -2322,10 +2322,10 @@
         <v>0</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>615.6</v>
+        <v>0</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>551.99</v>
+        <v>0</v>
       </c>
       <c r="J31" s="2" t="n">
         <v>0</v>
@@ -2337,7 +2337,7 @@
         <v>0</v>
       </c>
       <c r="M31" s="2" t="n">
-        <v>5710.6</v>
+        <v>0</v>
       </c>
       <c r="N31" s="2" t="n">
         <v>0</v>
@@ -2363,7 +2363,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>MENA COSTA GUIDO LENNIN</t>
+          <t>MEGGA-FRANK SAS</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
@@ -2382,10 +2382,10 @@
         <v>0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>0</v>
+        <v>615.6</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>0</v>
+        <v>551.99</v>
       </c>
       <c r="J32" s="2" t="n">
         <v>0</v>
@@ -2397,7 +2397,7 @@
         <v>0</v>
       </c>
       <c r="M32" s="2" t="n">
-        <v>0</v>
+        <v>5710.6</v>
       </c>
       <c r="N32" s="2" t="n">
         <v>0</v>
@@ -2423,7 +2423,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>MENESES TORRES OSCAR LEONARDO</t>
+          <t>MENA COSTA GUIDO LENNIN</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>MIM CONSTRUFERRETERIA E IMPORTADORA SAS</t>
+          <t>MENESES TORRES OSCAR LEONARDO</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
@@ -2543,7 +2543,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>MONTAÑO JIMENEZ SANDRA GABRIELA</t>
+          <t>MIM CONSTRUFERRETERIA E IMPORTADORA SAS</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
@@ -2603,7 +2603,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>MORALES GRACIELA ENITH</t>
+          <t>MONTAÑO JIMENEZ SANDRA GABRIELA</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
@@ -2663,7 +2663,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>MOROCHO BACUILIMA HILDA INES</t>
+          <t>MORALES GRACIELA ENITH</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
@@ -2723,7 +2723,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>MULLO GUACHO ANA LUCIA</t>
+          <t>MOROCHO BACUILIMA HILDA INES</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>OCHOA OCAMPO JOHANNA SUSANA</t>
+          <t>MULLO GUACHO ANA LUCIA</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
@@ -2820,7 +2820,7 @@
         <v>0</v>
       </c>
       <c r="N39" s="2" t="n">
-        <v>685.8</v>
+        <v>0</v>
       </c>
       <c r="O39" s="2" t="n">
         <v>0</v>
@@ -2843,7 +2843,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>ORTIZ GRANDA ANDREA DEL CISNE</t>
+          <t>OCHOA OCAMPO JOHANNA SUSANA</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
@@ -2880,7 +2880,7 @@
         <v>0</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>0</v>
+        <v>685.8</v>
       </c>
       <c r="O40" s="2" t="n">
         <v>0</v>
@@ -2903,7 +2903,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>PAUTA ASTUDILLO JULIO HERNAN</t>
+          <t>ORTIZ GRANDA ANDREA DEL CISNE</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
@@ -2937,7 +2937,7 @@
         <v>0</v>
       </c>
       <c r="M41" s="2" t="n">
-        <v>4867.08</v>
+        <v>0</v>
       </c>
       <c r="N41" s="2" t="n">
         <v>0</v>
@@ -2963,7 +2963,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>QUIÑONEZ LEON MARIA PURIFICACION</t>
+          <t>PAUTA ASTUDILLO JULIO HERNAN</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
@@ -2997,7 +2997,7 @@
         <v>0</v>
       </c>
       <c r="M42" s="2" t="n">
-        <v>0</v>
+        <v>4867.08</v>
       </c>
       <c r="N42" s="2" t="n">
         <v>0</v>
@@ -3023,7 +3023,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>REYES GUILLEN VICTOR EUGENIO</t>
+          <t>QUIÑONEZ LEON MARIA PURIFICACION</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
@@ -3083,7 +3083,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>ROBLES CAMPOVERDE TANIA CRISTINA</t>
+          <t>REYES GUILLEN VICTOR EUGENIO</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
@@ -3143,7 +3143,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>ROCAFUERTE LOPEZ EVELYN ESTEFANIA</t>
+          <t>ROBLES CAMPOVERDE TANIA CRISTINA</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
@@ -3203,7 +3203,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>RUALES SARAGURO JIMMY JAVIER</t>
+          <t>ROCAFUERTE LOPEZ EVELYN ESTEFANIA</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
@@ -3237,7 +3237,7 @@
         <v>0</v>
       </c>
       <c r="M46" s="2" t="n">
-        <v>508.04</v>
+        <v>0</v>
       </c>
       <c r="N46" s="2" t="n">
         <v>0</v>
@@ -3263,7 +3263,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>SANDOVAL GONZALEZ LAUTARO MARCELO</t>
+          <t>RUALES SARAGURO JIMMY JAVIER</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
@@ -3297,7 +3297,7 @@
         <v>0</v>
       </c>
       <c r="M47" s="2" t="n">
-        <v>0</v>
+        <v>508.04</v>
       </c>
       <c r="N47" s="2" t="n">
         <v>0</v>
@@ -3323,7 +3323,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>SANDOVAL GONZALEZ NILO GUILLERMO</t>
+          <t>SANDOVAL GONZALEZ LAUTARO MARCELO</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
@@ -3383,7 +3383,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>SANDOVAL MONTAÑO MARICELA DEL CISNE</t>
+          <t>SANDOVAL GONZALEZ NILO GUILLERMO</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
@@ -3443,7 +3443,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>SARITAMA HERRERA MARIA ELIZABETH</t>
+          <t>SANDOVAL MONTAÑO MARICELA DEL CISNE</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
@@ -3477,7 +3477,7 @@
         <v>0</v>
       </c>
       <c r="M50" s="2" t="n">
-        <v>71.11</v>
+        <v>0</v>
       </c>
       <c r="N50" s="2" t="n">
         <v>0</v>
@@ -3503,7 +3503,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>SARMIENTO SARMIENTO SANDRA EULALIA</t>
+          <t>SARITAMA HERRERA MARIA ELIZABETH</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
@@ -3513,7 +3513,7 @@
         <v>0</v>
       </c>
       <c r="E51" s="2" t="n">
-        <v>205.95</v>
+        <v>0</v>
       </c>
       <c r="F51" s="2" t="n">
         <v>0</v>
@@ -3537,7 +3537,7 @@
         <v>0</v>
       </c>
       <c r="M51" s="2" t="n">
-        <v>1550.24</v>
+        <v>71.11</v>
       </c>
       <c r="N51" s="2" t="n">
         <v>0</v>
@@ -3563,7 +3563,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>SIMANCAS AGUILAR HONORIO ANTONIO</t>
+          <t>SARMIENTO SARMIENTO SANDRA EULALIA</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
@@ -3573,7 +3573,7 @@
         <v>0</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>0</v>
+        <v>205.95</v>
       </c>
       <c r="F52" s="2" t="n">
         <v>0</v>
@@ -3597,7 +3597,7 @@
         <v>0</v>
       </c>
       <c r="M52" s="2" t="n">
-        <v>0</v>
+        <v>1550.24</v>
       </c>
       <c r="N52" s="2" t="n">
         <v>0</v>
@@ -3623,7 +3623,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>SOPLIN MENDOZA TABITA</t>
+          <t>SIMANCAS AGUILAR HONORIO ANTONIO</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
@@ -3683,7 +3683,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>TAMAY SANTACRUZ MARIA ANGELICA</t>
+          <t>SOPLIN MENDOZA TABITA</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
@@ -3743,7 +3743,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
+          <t>TAMAY SANTACRUZ MARIA ANGELICA</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
@@ -3803,7 +3803,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>VEINTIMILLA JARAMILLO HERMANOS VJHNOS S.A.S.</t>
+          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
@@ -3863,7 +3863,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>VERA CABRERA JORGE ENRIQUE</t>
+          <t>VEINTIMILLA JARAMILLO HERMANOS VJHNOS S.A.S.</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
@@ -3923,137 +3923,197 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
+          <t>VERA CABRERA JORGE ENRIQUE</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D58" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E58" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F58" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G58" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H58" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I58" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J58" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K58" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L58" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M58" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N58" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O58" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P58" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q58" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R58" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
           <t>VIVANCO MALDONADO SILVANA MARILY</t>
         </is>
       </c>
-      <c r="C58" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D58" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E58" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F58" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G58" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H58" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I58" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J58" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K58" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L58" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M58" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N58" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O58" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P58" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q58" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R58" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="C59" s="3" t="inlineStr">
-        <is>
-          <t>0 de 57</t>
-        </is>
-      </c>
-      <c r="D59" s="3" t="inlineStr">
-        <is>
-          <t>1 de 57</t>
-        </is>
-      </c>
-      <c r="E59" s="3" t="inlineStr">
-        <is>
-          <t>3 de 57</t>
-        </is>
-      </c>
-      <c r="F59" s="3" t="inlineStr">
-        <is>
-          <t>0 de 57</t>
-        </is>
-      </c>
-      <c r="G59" s="3" t="inlineStr">
-        <is>
-          <t>0 de 57</t>
-        </is>
-      </c>
-      <c r="H59" s="3" t="inlineStr">
-        <is>
-          <t>4 de 57</t>
-        </is>
-      </c>
-      <c r="I59" s="3" t="inlineStr">
-        <is>
-          <t>4 de 57</t>
-        </is>
-      </c>
-      <c r="J59" s="3" t="inlineStr">
-        <is>
-          <t>0 de 57</t>
-        </is>
-      </c>
-      <c r="K59" s="3" t="inlineStr">
-        <is>
-          <t>2 de 57</t>
-        </is>
-      </c>
-      <c r="L59" s="3" t="inlineStr">
-        <is>
-          <t>0 de 57</t>
-        </is>
-      </c>
-      <c r="M59" s="3" t="inlineStr">
-        <is>
-          <t>10 de 57</t>
-        </is>
-      </c>
-      <c r="N59" s="3" t="inlineStr">
-        <is>
-          <t>1 de 57</t>
-        </is>
-      </c>
-      <c r="O59" s="3" t="inlineStr">
-        <is>
-          <t>0 de 57</t>
-        </is>
-      </c>
-      <c r="P59" s="3" t="inlineStr">
-        <is>
-          <t>0 de 57</t>
-        </is>
-      </c>
-      <c r="Q59" s="3" t="inlineStr">
-        <is>
-          <t>0 de 57</t>
-        </is>
-      </c>
-      <c r="R59" s="3" t="inlineStr">
-        <is>
-          <t>0 de 57</t>
+      <c r="C59" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D59" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E59" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F59" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G59" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H59" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I59" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J59" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K59" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L59" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M59" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N59" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O59" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P59" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q59" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R59" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>0 de 58</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>1 de 58</t>
+        </is>
+      </c>
+      <c r="E60" s="3" t="inlineStr">
+        <is>
+          <t>3 de 58</t>
+        </is>
+      </c>
+      <c r="F60" s="3" t="inlineStr">
+        <is>
+          <t>0 de 58</t>
+        </is>
+      </c>
+      <c r="G60" s="3" t="inlineStr">
+        <is>
+          <t>0 de 58</t>
+        </is>
+      </c>
+      <c r="H60" s="3" t="inlineStr">
+        <is>
+          <t>4 de 58</t>
+        </is>
+      </c>
+      <c r="I60" s="3" t="inlineStr">
+        <is>
+          <t>4 de 58</t>
+        </is>
+      </c>
+      <c r="J60" s="3" t="inlineStr">
+        <is>
+          <t>0 de 58</t>
+        </is>
+      </c>
+      <c r="K60" s="3" t="inlineStr">
+        <is>
+          <t>2 de 58</t>
+        </is>
+      </c>
+      <c r="L60" s="3" t="inlineStr">
+        <is>
+          <t>0 de 58</t>
+        </is>
+      </c>
+      <c r="M60" s="3" t="inlineStr">
+        <is>
+          <t>11 de 58</t>
+        </is>
+      </c>
+      <c r="N60" s="3" t="inlineStr">
+        <is>
+          <t>1 de 58</t>
+        </is>
+      </c>
+      <c r="O60" s="3" t="inlineStr">
+        <is>
+          <t>0 de 58</t>
+        </is>
+      </c>
+      <c r="P60" s="3" t="inlineStr">
+        <is>
+          <t>0 de 58</t>
+        </is>
+      </c>
+      <c r="Q60" s="3" t="inlineStr">
+        <is>
+          <t>0 de 58</t>
+        </is>
+      </c>
+      <c r="R60" s="3" t="inlineStr">
+        <is>
+          <t>0 de 58</t>
         </is>
       </c>
     </row>
@@ -4068,7 +4128,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G53"/>
+  <dimension ref="A1:G54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4179,7 +4239,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ALTAMIRANO VILLAVICENCIO JUAN ALEJANDRO</t>
+          <t>ALTAMIRANO MARCATOMA MARIA ANA</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
@@ -4192,10 +4252,10 @@
         <v>0</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>0</v>
+        <v>1361.84</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -4206,7 +4266,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ALVAREZ SAAVEDRA EDWIN GEOVANNY</t>
+          <t>ALTAMIRANO VILLAVICENCIO JUAN ALEJANDRO</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
@@ -4222,7 +4282,7 @@
         <v>0</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="6">
@@ -4233,7 +4293,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ANGAMARCA CURIPOMA JENNY MARIA</t>
+          <t>ALVAREZ SAAVEDRA EDWIN GEOVANNY</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
@@ -4260,14 +4320,14 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ARIAS CARDENAS BOLIVAR MAURICIO</t>
+          <t>ANGAMARCA CURIPOMA JENNY MARIA</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>1049.69</v>
+        <v>0</v>
       </c>
       <c r="E7" s="2" t="n">
         <v>0</v>
@@ -4276,7 +4336,7 @@
         <v>0</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -4287,23 +4347,23 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ARMIJOS SALINAS LUIS CLAUDIO</t>
+          <t>ARIAS CARDENAS BOLIVAR MAURICIO</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>1284.32</v>
+        <v>1049.69</v>
       </c>
       <c r="E8" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>708.88</v>
+        <v>0</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>1000</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="9">
@@ -4314,23 +4374,23 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ASES GAVILANEZ FAUSTO HERNAN</t>
+          <t>ARMIJOS SALINAS LUIS CLAUDIO</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0</v>
+        <v>1284.32</v>
       </c>
       <c r="E9" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>0</v>
+        <v>708.88</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="10">
@@ -4341,7 +4401,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>BARROS YUNGA DIEGO VINICIO</t>
+          <t>ASES GAVILANEZ FAUSTO HERNAN</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
@@ -4354,10 +4414,10 @@
         <v>0</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>620.73</v>
+        <v>0</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -4368,7 +4428,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>BRITO CARDENAS RUTH CECILIA</t>
+          <t>BARROS YUNGA DIEGO VINICIO</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
@@ -4381,10 +4441,10 @@
         <v>0</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>0</v>
+        <v>620.73</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>0</v>
+        <v>500</v>
       </c>
     </row>
     <row r="12">
@@ -4395,23 +4455,23 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>CARRION MORALES CARLOS ENRIQUE</t>
+          <t>BRITO CARDENAS RUTH CECILIA</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>50.54</v>
+        <v>0</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>258.49</v>
+        <v>0</v>
       </c>
       <c r="F12" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -4422,23 +4482,23 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>COMERCIAL LUNA PAZMIÑO CIA. LTDA.</t>
+          <t>CARRION MORALES CARLOS ENRIQUE</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>0</v>
+        <v>50.54</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>0</v>
+        <v>258.49</v>
       </c>
       <c r="F13" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>0</v>
+        <v>500</v>
       </c>
     </row>
     <row r="14">
@@ -4449,23 +4509,23 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>CORONEL PINOS CLARA MARIA</t>
+          <t>COMERCIAL LUNA PAZMIÑO CIA. LTDA.</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>2068.01</v>
+        <v>0</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>5446.06</v>
+        <v>0</v>
       </c>
       <c r="F14" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>1500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -4476,20 +4536,20 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>CORPORACION AREVALO-YUMBLA E HIJOS</t>
+          <t>CORONEL PINOS CLARA MARIA</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>0</v>
+        <v>2068.01</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>0</v>
+        <v>5446.06</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>1214.7</v>
+        <v>0</v>
       </c>
       <c r="G15" s="2" t="n">
         <v>1500</v>
@@ -4503,7 +4563,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>DIAZ CHAVEZ DIEGO FERNANDO</t>
+          <t>CORPORACION AREVALO-YUMBLA E HIJOS</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
@@ -4516,10 +4576,10 @@
         <v>0</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>0</v>
+        <v>1214.7</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>0</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="17">
@@ -4530,7 +4590,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>DISTRIBUIDORA VASQUEZ ORDOÑEZ DISTRIVASOR CIA LTDA</t>
+          <t>DIAZ CHAVEZ DIEGO FERNANDO</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
@@ -4546,7 +4606,7 @@
         <v>0</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -4557,14 +4617,14 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>ESPINOZA GOMEZ LILIA ROSARIO</t>
+          <t>DISTRIBUIDORA VASQUEZ ORDOÑEZ DISTRIVASOR CIA LTDA</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>3072.2</v>
+        <v>0</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>426.67</v>
+        <v>0</v>
       </c>
       <c r="E18" s="2" t="n">
         <v>0</v>
@@ -4573,7 +4633,7 @@
         <v>0</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>3000</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="19">
@@ -4584,23 +4644,23 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>FABIMP BENIGNO BRAVO S.A.S.</t>
+          <t>ESPINOZA GOMEZ LILIA ROSARIO</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>0</v>
+        <v>3072.2</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>3603.22</v>
+        <v>426.67</v>
       </c>
       <c r="E19" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>6241.39</v>
+        <v>0</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>2000</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="20">
@@ -4611,23 +4671,23 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>FERRICENTER EL ARENAL CIA. LTDA.</t>
+          <t>FABIMP BENIGNO BRAVO S.A.S.</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>4096.36</v>
+        <v>0</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>0</v>
+        <v>3603.22</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>1550.24</v>
+        <v>0</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>0</v>
+        <v>6241.39</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>1500</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="21">
@@ -4638,23 +4698,23 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>GLOBAL MOYANO &amp; ASOCIADOS LEMO S.A.S.</t>
+          <t>FERRICENTER EL ARENAL CIA. LTDA.</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>70.37</v>
+        <v>4096.36</v>
       </c>
       <c r="D21" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>0</v>
+        <v>1550.24</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>19.66</v>
+        <v>0</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>0</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="22">
@@ -4665,20 +4725,20 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>GRANDA SANDOVAL JACKELINE ELIZABETH</t>
+          <t>GLOBAL MOYANO &amp; ASOCIADOS LEMO S.A.S.</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>0</v>
+        <v>70.37</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>1045.76</v>
+        <v>0</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>68.23</v>
+        <v>0</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>0</v>
+        <v>19.66</v>
       </c>
       <c r="G22" s="2" t="n">
         <v>0</v>
@@ -4692,23 +4752,23 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>HUERTA MUÑOZ NANCY ELIZABETH</t>
+          <t>GRANDA SANDOVAL JACKELINE ELIZABETH</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>4922.83</v>
+        <v>0</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>0</v>
+        <v>1045.76</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>1499.16</v>
+        <v>68.23</v>
       </c>
       <c r="F23" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
@@ -4719,23 +4779,23 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>IMPORTADORA ORTEGA CIA. LTDA.</t>
+          <t>HUERTA MUÑOZ NANCY ELIZABETH</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>0</v>
+        <v>4922.83</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>1479.64</v>
+        <v>0</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>11932.7</v>
+        <v>1499.16</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>7610.19</v>
+        <v>0</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>4000</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="25">
@@ -4746,23 +4806,23 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>JIMBO BRITO SELENE PATRICIA</t>
+          <t>IMPORTADORA ORTEGA CIA. LTDA.</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>0</v>
+        <v>1479.64</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>0</v>
+        <v>11932.7</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>5097.28</v>
+        <v>7610.19</v>
       </c>
       <c r="G25" s="2" t="n">
-        <v>0</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="26">
@@ -4773,7 +4833,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>JIMENEZ GORDILLO LADY KARINA</t>
+          <t>JIMBO BRITO SELENE PATRICIA</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
@@ -4786,7 +4846,7 @@
         <v>0</v>
       </c>
       <c r="F26" s="2" t="n">
-        <v>0</v>
+        <v>5097.28</v>
       </c>
       <c r="G26" s="2" t="n">
         <v>0</v>
@@ -4800,7 +4860,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>JUAREZ FLORES JORGE WILLIAMS</t>
+          <t>JIMENEZ GORDILLO LADY KARINA</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
@@ -4827,11 +4887,11 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>LEMA ESPINOZA MANUEL MARIA</t>
+          <t>JUAREZ FLORES JORGE WILLIAMS</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>865.47</v>
+        <v>0</v>
       </c>
       <c r="D28" s="2" t="n">
         <v>0</v>
@@ -4843,7 +4903,7 @@
         <v>0</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
@@ -4854,11 +4914,11 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>MEGGA-FRANK SAS</t>
+          <t>LEMA ESPINOZA MANUEL MARIA</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>0</v>
+        <v>865.47</v>
       </c>
       <c r="D29" s="2" t="n">
         <v>0</v>
@@ -4867,10 +4927,10 @@
         <v>0</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>6878.19</v>
+        <v>0</v>
       </c>
       <c r="G29" s="2" t="n">
-        <v>5000</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="30">
@@ -4881,7 +4941,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>MENA COSTA GUIDO LENNIN</t>
+          <t>MEGGA-FRANK SAS</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
@@ -4894,10 +4954,10 @@
         <v>0</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>0</v>
+        <v>6878.19</v>
       </c>
       <c r="G30" s="2" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="31">
@@ -4908,14 +4968,14 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>MENESES TORRES OSCAR LEONARDO</t>
+          <t>MENA COSTA GUIDO LENNIN</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>401.57</v>
+        <v>0</v>
       </c>
       <c r="E31" s="2" t="n">
         <v>0</v>
@@ -4924,7 +4984,7 @@
         <v>0</v>
       </c>
       <c r="G31" s="2" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
@@ -4935,23 +4995,23 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>MIM CONSTRUFERRETERIA E IMPORTADORA SAS</t>
+          <t>MENESES TORRES OSCAR LEONARDO</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D32" s="2" t="n">
-        <v>0</v>
+        <v>401.57</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>4583.45</v>
+        <v>0</v>
       </c>
       <c r="F32" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G32" s="2" t="n">
-        <v>2000</v>
+        <v>500</v>
       </c>
     </row>
     <row r="33">
@@ -4962,7 +5022,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>MONTAÑO JIMENEZ SANDRA GABRIELA</t>
+          <t>MIM CONSTRUFERRETERIA E IMPORTADORA SAS</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
@@ -4972,13 +5032,13 @@
         <v>0</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>1094</v>
+        <v>4583.45</v>
       </c>
       <c r="F33" s="2" t="n">
-        <v>37.75</v>
+        <v>0</v>
       </c>
       <c r="G33" s="2" t="n">
-        <v>0</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="34">
@@ -4989,20 +5049,20 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>MOROCHO BACUILIMA HILDA INES</t>
+          <t>MONTAÑO JIMENEZ SANDRA GABRIELA</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
-        <v>16.74</v>
+        <v>0</v>
       </c>
       <c r="D34" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>1133.57</v>
+        <v>1094</v>
       </c>
       <c r="F34" s="2" t="n">
-        <v>0</v>
+        <v>37.75</v>
       </c>
       <c r="G34" s="2" t="n">
         <v>0</v>
@@ -5016,17 +5076,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>MULLO GUACHO ANA LUCIA</t>
+          <t>MOROCHO BACUILIMA HILDA INES</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
-        <v>0</v>
+        <v>16.74</v>
       </c>
       <c r="D35" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>0</v>
+        <v>1133.57</v>
       </c>
       <c r="F35" s="2" t="n">
         <v>0</v>
@@ -5043,20 +5103,20 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>OCHOA OCAMPO JOHANNA SUSANA</t>
+          <t>MULLO GUACHO ANA LUCIA</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D36" s="2" t="n">
-        <v>976.9400000000001</v>
+        <v>0</v>
       </c>
       <c r="E36" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>685.8</v>
+        <v>0</v>
       </c>
       <c r="G36" s="2" t="n">
         <v>0</v>
@@ -5070,23 +5130,23 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>PAUTA ASTUDILLO JULIO HERNAN</t>
+          <t>OCHOA OCAMPO JOHANNA SUSANA</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D37" s="2" t="n">
-        <v>321.93</v>
+        <v>976.9400000000001</v>
       </c>
       <c r="E37" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F37" s="2" t="n">
-        <v>4867.08</v>
+        <v>685.8</v>
       </c>
       <c r="G37" s="2" t="n">
-        <v>1500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38">
@@ -5097,23 +5157,23 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>QUIÑONEZ LEON MARIA PURIFICACION</t>
+          <t>PAUTA ASTUDILLO JULIO HERNAN</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D38" s="2" t="n">
-        <v>0</v>
+        <v>321.93</v>
       </c>
       <c r="E38" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>0</v>
+        <v>4867.08</v>
       </c>
       <c r="G38" s="2" t="n">
-        <v>0</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="39">
@@ -5124,11 +5184,11 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>REYES GUILLEN VICTOR EUGENIO</t>
+          <t>QUIÑONEZ LEON MARIA PURIFICACION</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
-        <v>1882.6</v>
+        <v>0</v>
       </c>
       <c r="D39" s="2" t="n">
         <v>0</v>
@@ -5137,7 +5197,7 @@
         <v>0</v>
       </c>
       <c r="F39" s="2" t="n">
-        <v>4.06</v>
+        <v>0</v>
       </c>
       <c r="G39" s="2" t="n">
         <v>0</v>
@@ -5151,23 +5211,23 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>ROBLES CAMPOVERDE TANIA CRISTINA</t>
+          <t>REYES GUILLEN VICTOR EUGENIO</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
-        <v>101.16</v>
+        <v>1882.6</v>
       </c>
       <c r="D40" s="2" t="n">
-        <v>2180.13</v>
+        <v>0</v>
       </c>
       <c r="E40" s="2" t="n">
-        <v>3085.71</v>
+        <v>0</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>0</v>
+        <v>4.06</v>
       </c>
       <c r="G40" s="2" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41">
@@ -5178,23 +5238,23 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>ROCAFUERTE LOPEZ EVELYN ESTEFANIA</t>
+          <t>ROBLES CAMPOVERDE TANIA CRISTINA</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
-        <v>0</v>
+        <v>101.16</v>
       </c>
       <c r="D41" s="2" t="n">
-        <v>0</v>
+        <v>2180.13</v>
       </c>
       <c r="E41" s="2" t="n">
-        <v>0</v>
+        <v>3085.71</v>
       </c>
       <c r="F41" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G41" s="2" t="n">
-        <v>0</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="42">
@@ -5205,23 +5265,23 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>RUALES SARAGURO JIMMY JAVIER</t>
+          <t>ROCAFUERTE LOPEZ EVELYN ESTEFANIA</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
-        <v>9109.299999999999</v>
+        <v>0</v>
       </c>
       <c r="D42" s="2" t="n">
-        <v>5577.51</v>
+        <v>0</v>
       </c>
       <c r="E42" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F42" s="2" t="n">
-        <v>547.6900000000001</v>
+        <v>0</v>
       </c>
       <c r="G42" s="2" t="n">
-        <v>5000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43">
@@ -5232,23 +5292,23 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>SANDOVAL GONZALEZ NILO GUILLERMO</t>
+          <t>RUALES SARAGURO JIMMY JAVIER</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
-        <v>0</v>
+        <v>9109.299999999999</v>
       </c>
       <c r="D43" s="2" t="n">
-        <v>1432.86</v>
+        <v>5577.51</v>
       </c>
       <c r="E43" s="2" t="n">
-        <v>-1284.32</v>
+        <v>0</v>
       </c>
       <c r="F43" s="2" t="n">
-        <v>0</v>
+        <v>547.6900000000001</v>
       </c>
       <c r="G43" s="2" t="n">
-        <v>1200</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="44">
@@ -5259,23 +5319,23 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>SARITAMA HERRERA MARIA ELIZABETH</t>
+          <t>SANDOVAL GONZALEZ NILO GUILLERMO</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D44" s="2" t="n">
-        <v>0</v>
+        <v>1432.86</v>
       </c>
       <c r="E44" s="2" t="n">
-        <v>474.08</v>
+        <v>-1284.32</v>
       </c>
       <c r="F44" s="2" t="n">
-        <v>71.11</v>
+        <v>0</v>
       </c>
       <c r="G44" s="2" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="45">
@@ -5286,7 +5346,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>SARMIENTO SARMIENTO SANDRA EULALIA</t>
+          <t>SARITAMA HERRERA MARIA ELIZABETH</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
@@ -5296,13 +5356,13 @@
         <v>0</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>0</v>
+        <v>474.08</v>
       </c>
       <c r="F45" s="2" t="n">
-        <v>1756.19</v>
+        <v>71.11</v>
       </c>
       <c r="G45" s="2" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46">
@@ -5313,23 +5373,23 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>SIMANCAS AGUILAR HONORIO ANTONIO</t>
+          <t>SARMIENTO SARMIENTO SANDRA EULALIA</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
-        <v>3155.46</v>
+        <v>0</v>
       </c>
       <c r="D46" s="2" t="n">
-        <v>1348.76</v>
+        <v>0</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>13692.06</v>
+        <v>0</v>
       </c>
       <c r="F46" s="2" t="n">
-        <v>0</v>
+        <v>1756.19</v>
       </c>
       <c r="G46" s="2" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="47">
@@ -5340,17 +5400,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>SOPLIN MENDOZA TABITA</t>
+          <t>SIMANCAS AGUILAR HONORIO ANTONIO</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
-        <v>0</v>
+        <v>3155.46</v>
       </c>
       <c r="D47" s="2" t="n">
-        <v>0</v>
+        <v>1348.76</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>0</v>
+        <v>13692.06</v>
       </c>
       <c r="F47" s="2" t="n">
         <v>0</v>
@@ -5367,11 +5427,11 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>TAMAY SANTACRUZ MARIA ANGELICA</t>
+          <t>SOPLIN MENDOZA TABITA</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
-        <v>4237.6</v>
+        <v>0</v>
       </c>
       <c r="D48" s="2" t="n">
         <v>0</v>
@@ -5380,10 +5440,10 @@
         <v>0</v>
       </c>
       <c r="F48" s="2" t="n">
-        <v>37.75</v>
+        <v>0</v>
       </c>
       <c r="G48" s="2" t="n">
-        <v>1500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49">
@@ -5394,11 +5454,11 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
+          <t>TAMAY SANTACRUZ MARIA ANGELICA</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
-        <v>0</v>
+        <v>4237.6</v>
       </c>
       <c r="D49" s="2" t="n">
         <v>0</v>
@@ -5407,10 +5467,10 @@
         <v>0</v>
       </c>
       <c r="F49" s="2" t="n">
-        <v>0</v>
+        <v>37.75</v>
       </c>
       <c r="G49" s="2" t="n">
-        <v>2000</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="50">
@@ -5421,7 +5481,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>VEINTIMILLA JARAMILLO HERMANOS VJHNOS S.A.S.</t>
+          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
@@ -5437,7 +5497,7 @@
         <v>0</v>
       </c>
       <c r="G50" s="2" t="n">
-        <v>0</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="51">
@@ -5448,7 +5508,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>VERA CABRERA JORGE ENRIQUE</t>
+          <t>VEINTIMILLA JARAMILLO HERMANOS VJHNOS S.A.S.</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
@@ -5475,39 +5535,66 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
+          <t>VERA CABRERA JORGE ENRIQUE</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D52" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E52" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F52" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G52" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
           <t>VIVANCO MALDONADO SILVANA MARILY</t>
         </is>
       </c>
-      <c r="C52" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D52" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E52" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F52" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G52" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="C53" s="4" t="n">
+      <c r="C53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G53" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="C54" s="4" t="n">
         <v>35603.86</v>
       </c>
-      <c r="D53" s="4" t="n">
+      <c r="D54" s="4" t="n">
         <v>28143.93</v>
       </c>
-      <c r="E53" s="4" t="n">
+      <c r="E54" s="4" t="n">
         <v>43533.43</v>
       </c>
-      <c r="F53" s="4" t="n">
-        <v>36408.6</v>
-      </c>
-      <c r="G53" s="4" t="n">
+      <c r="F54" s="4" t="n">
+        <v>37770.44</v>
+      </c>
+      <c r="G54" s="4" t="n">
         <v>47200</v>
       </c>
     </row>
@@ -5528,7 +5615,7 @@
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
     <col width="25" customWidth="1" min="6" max="6"/>
   </cols>
@@ -5604,13 +5691,13 @@
         <v>4001</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>75.5</v>
+        <v>108.9</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>3925.5</v>
+        <v>3892.1</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>0.01887028242939265</v>
+        <v>0.02721819545113722</v>
       </c>
     </row>
     <row r="4">
@@ -5820,13 +5907,13 @@
         <v>39603</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>27361.86</v>
+        <v>28690.3</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>12241.14</v>
+        <v>10912.7</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0.6909037194151958</v>
+        <v>0.7244476428553392</v>
       </c>
     </row>
     <row r="13">
@@ -5839,13 +5926,13 @@
         <v>49040.76</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>36474.39</v>
+        <v>37836.23</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>12566.37</v>
+        <v>11204.53</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>0.7437566220425621</v>
+        <v>0.7715261753692234</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-25 16:30:18
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R60"/>
+  <dimension ref="A1:R61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2363,7 +2363,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>MEGGA-FRANK SAS</t>
+          <t>MARIN SANCHEZ GABRIEL ALEXANDER</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
@@ -2382,22 +2382,22 @@
         <v>0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>615.6</v>
+        <v>0</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>551.99</v>
+        <v>184.95</v>
       </c>
       <c r="J32" s="2" t="n">
         <v>0</v>
       </c>
       <c r="K32" s="2" t="n">
-        <v>0</v>
+        <v>201.32</v>
       </c>
       <c r="L32" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M32" s="2" t="n">
-        <v>5710.6</v>
+        <v>0</v>
       </c>
       <c r="N32" s="2" t="n">
         <v>0</v>
@@ -2423,7 +2423,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>MENA COSTA GUIDO LENNIN</t>
+          <t>MEGGA-FRANK SAS</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
@@ -2442,10 +2442,10 @@
         <v>0</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>0</v>
+        <v>615.6</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>0</v>
+        <v>551.99</v>
       </c>
       <c r="J33" s="2" t="n">
         <v>0</v>
@@ -2457,7 +2457,7 @@
         <v>0</v>
       </c>
       <c r="M33" s="2" t="n">
-        <v>0</v>
+        <v>5710.6</v>
       </c>
       <c r="N33" s="2" t="n">
         <v>0</v>
@@ -2483,7 +2483,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>MENESES TORRES OSCAR LEONARDO</t>
+          <t>MENA COSTA GUIDO LENNIN</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
@@ -2543,7 +2543,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>MIM CONSTRUFERRETERIA E IMPORTADORA SAS</t>
+          <t>MENESES TORRES OSCAR LEONARDO</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
@@ -2603,7 +2603,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>MONTAÑO JIMENEZ SANDRA GABRIELA</t>
+          <t>MIM CONSTRUFERRETERIA E IMPORTADORA SAS</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
@@ -2663,7 +2663,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>MORALES GRACIELA ENITH</t>
+          <t>MONTAÑO JIMENEZ SANDRA GABRIELA</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
@@ -2723,7 +2723,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>MOROCHO BACUILIMA HILDA INES</t>
+          <t>MORALES GRACIELA ENITH</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>MULLO GUACHO ANA LUCIA</t>
+          <t>MOROCHO BACUILIMA HILDA INES</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
@@ -2843,7 +2843,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>OCHOA OCAMPO JOHANNA SUSANA</t>
+          <t>MULLO GUACHO ANA LUCIA</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
@@ -2871,7 +2871,7 @@
         <v>0</v>
       </c>
       <c r="K40" s="2" t="n">
-        <v>367.08</v>
+        <v>0</v>
       </c>
       <c r="L40" s="2" t="n">
         <v>0</v>
@@ -2880,7 +2880,7 @@
         <v>0</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>685.8</v>
+        <v>0</v>
       </c>
       <c r="O40" s="2" t="n">
         <v>0</v>
@@ -2903,7 +2903,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>ORTIZ GRANDA ANDREA DEL CISNE</t>
+          <t>OCHOA OCAMPO JOHANNA SUSANA</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
@@ -2931,7 +2931,7 @@
         <v>0</v>
       </c>
       <c r="K41" s="2" t="n">
-        <v>0</v>
+        <v>367.08</v>
       </c>
       <c r="L41" s="2" t="n">
         <v>0</v>
@@ -2940,7 +2940,7 @@
         <v>0</v>
       </c>
       <c r="N41" s="2" t="n">
-        <v>0</v>
+        <v>685.8</v>
       </c>
       <c r="O41" s="2" t="n">
         <v>0</v>
@@ -2963,7 +2963,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>PAUTA ASTUDILLO JULIO HERNAN</t>
+          <t>ORTIZ GRANDA ANDREA DEL CISNE</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
@@ -2997,7 +2997,7 @@
         <v>0</v>
       </c>
       <c r="M42" s="2" t="n">
-        <v>4867.08</v>
+        <v>0</v>
       </c>
       <c r="N42" s="2" t="n">
         <v>0</v>
@@ -3023,7 +3023,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>QUIÑONEZ LEON MARIA PURIFICACION</t>
+          <t>PAUTA ASTUDILLO JULIO HERNAN</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
@@ -3057,7 +3057,7 @@
         <v>0</v>
       </c>
       <c r="M43" s="2" t="n">
-        <v>0</v>
+        <v>4867.08</v>
       </c>
       <c r="N43" s="2" t="n">
         <v>0</v>
@@ -3083,7 +3083,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>REYES GUILLEN VICTOR EUGENIO</t>
+          <t>QUIÑONEZ LEON MARIA PURIFICACION</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
@@ -3143,7 +3143,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>ROBLES CAMPOVERDE TANIA CRISTINA</t>
+          <t>REYES GUILLEN VICTOR EUGENIO</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
@@ -3203,7 +3203,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>ROCAFUERTE LOPEZ EVELYN ESTEFANIA</t>
+          <t>ROBLES CAMPOVERDE TANIA CRISTINA</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
@@ -3263,7 +3263,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>RUALES SARAGURO JIMMY JAVIER</t>
+          <t>ROCAFUERTE LOPEZ EVELYN ESTEFANIA</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
@@ -3297,7 +3297,7 @@
         <v>0</v>
       </c>
       <c r="M47" s="2" t="n">
-        <v>926.02</v>
+        <v>0</v>
       </c>
       <c r="N47" s="2" t="n">
         <v>0</v>
@@ -3323,7 +3323,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>SANDOVAL GONZALEZ LAUTARO MARCELO</t>
+          <t>RUALES SARAGURO JIMMY JAVIER</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
@@ -3357,7 +3357,7 @@
         <v>0</v>
       </c>
       <c r="M48" s="2" t="n">
-        <v>0</v>
+        <v>926.02</v>
       </c>
       <c r="N48" s="2" t="n">
         <v>0</v>
@@ -3383,7 +3383,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>SANDOVAL GONZALEZ NILO GUILLERMO</t>
+          <t>SANDOVAL GONZALEZ LAUTARO MARCELO</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
@@ -3443,7 +3443,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>SANDOVAL MONTAÑO MARICELA DEL CISNE</t>
+          <t>SANDOVAL GONZALEZ NILO GUILLERMO</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
@@ -3503,7 +3503,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>SARITAMA HERRERA MARIA ELIZABETH</t>
+          <t>SANDOVAL MONTAÑO MARICELA DEL CISNE</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
@@ -3537,7 +3537,7 @@
         <v>0</v>
       </c>
       <c r="M51" s="2" t="n">
-        <v>71.11</v>
+        <v>0</v>
       </c>
       <c r="N51" s="2" t="n">
         <v>0</v>
@@ -3563,7 +3563,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>SARMIENTO SARMIENTO SANDRA EULALIA</t>
+          <t>SARITAMA HERRERA MARIA ELIZABETH</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
@@ -3573,7 +3573,7 @@
         <v>0</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>205.95</v>
+        <v>0</v>
       </c>
       <c r="F52" s="2" t="n">
         <v>0</v>
@@ -3597,7 +3597,7 @@
         <v>0</v>
       </c>
       <c r="M52" s="2" t="n">
-        <v>1550.24</v>
+        <v>71.11</v>
       </c>
       <c r="N52" s="2" t="n">
         <v>0</v>
@@ -3623,7 +3623,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>SIMANCAS AGUILAR HONORIO ANTONIO</t>
+          <t>SARMIENTO SARMIENTO SANDRA EULALIA</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
@@ -3633,7 +3633,7 @@
         <v>0</v>
       </c>
       <c r="E53" s="2" t="n">
-        <v>0</v>
+        <v>205.95</v>
       </c>
       <c r="F53" s="2" t="n">
         <v>0</v>
@@ -3657,7 +3657,7 @@
         <v>0</v>
       </c>
       <c r="M53" s="2" t="n">
-        <v>0</v>
+        <v>1550.24</v>
       </c>
       <c r="N53" s="2" t="n">
         <v>0</v>
@@ -3683,7 +3683,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>SOPLIN MENDOZA TABITA</t>
+          <t>SIMANCAS AGUILAR HONORIO ANTONIO</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
@@ -3743,7 +3743,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>TAMAY SANTACRUZ MARIA ANGELICA</t>
+          <t>SOPLIN MENDOZA TABITA</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
@@ -3803,7 +3803,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
+          <t>TAMAY SANTACRUZ MARIA ANGELICA</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
@@ -3863,7 +3863,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>VEINTIMILLA JARAMILLO HERMANOS VJHNOS S.A.S.</t>
+          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
@@ -3923,7 +3923,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>VERA CABRERA JORGE ENRIQUE</t>
+          <t>VEINTIMILLA JARAMILLO HERMANOS VJHNOS S.A.S.</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
@@ -3983,137 +3983,197 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
+          <t>VERA CABRERA JORGE ENRIQUE</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D59" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E59" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F59" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G59" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H59" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I59" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J59" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K59" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L59" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M59" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N59" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O59" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P59" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q59" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R59" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
           <t>VIVANCO MALDONADO SILVANA MARILY</t>
         </is>
       </c>
-      <c r="C59" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D59" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E59" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F59" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G59" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H59" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I59" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J59" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K59" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L59" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M59" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N59" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O59" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P59" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q59" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R59" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="C60" s="3" t="inlineStr">
-        <is>
-          <t>0 de 58</t>
-        </is>
-      </c>
-      <c r="D60" s="3" t="inlineStr">
-        <is>
-          <t>1 de 58</t>
-        </is>
-      </c>
-      <c r="E60" s="3" t="inlineStr">
-        <is>
-          <t>4 de 58</t>
-        </is>
-      </c>
-      <c r="F60" s="3" t="inlineStr">
-        <is>
-          <t>0 de 58</t>
-        </is>
-      </c>
-      <c r="G60" s="3" t="inlineStr">
-        <is>
-          <t>0 de 58</t>
-        </is>
-      </c>
-      <c r="H60" s="3" t="inlineStr">
-        <is>
-          <t>6 de 58</t>
-        </is>
-      </c>
-      <c r="I60" s="3" t="inlineStr">
-        <is>
-          <t>6 de 58</t>
-        </is>
-      </c>
-      <c r="J60" s="3" t="inlineStr">
-        <is>
-          <t>0 de 58</t>
-        </is>
-      </c>
-      <c r="K60" s="3" t="inlineStr">
-        <is>
-          <t>4 de 58</t>
-        </is>
-      </c>
-      <c r="L60" s="3" t="inlineStr">
-        <is>
-          <t>1 de 58</t>
-        </is>
-      </c>
-      <c r="M60" s="3" t="inlineStr">
-        <is>
-          <t>12 de 58</t>
-        </is>
-      </c>
-      <c r="N60" s="3" t="inlineStr">
-        <is>
-          <t>1 de 58</t>
-        </is>
-      </c>
-      <c r="O60" s="3" t="inlineStr">
-        <is>
-          <t>0 de 58</t>
-        </is>
-      </c>
-      <c r="P60" s="3" t="inlineStr">
-        <is>
-          <t>0 de 58</t>
-        </is>
-      </c>
-      <c r="Q60" s="3" t="inlineStr">
-        <is>
-          <t>0 de 58</t>
-        </is>
-      </c>
-      <c r="R60" s="3" t="inlineStr">
-        <is>
-          <t>0 de 58</t>
+      <c r="C60" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D60" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E60" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F60" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G60" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H60" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I60" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J60" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K60" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L60" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M60" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N60" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O60" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P60" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q60" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R60" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>0 de 59</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t>1 de 59</t>
+        </is>
+      </c>
+      <c r="E61" s="3" t="inlineStr">
+        <is>
+          <t>4 de 59</t>
+        </is>
+      </c>
+      <c r="F61" s="3" t="inlineStr">
+        <is>
+          <t>0 de 59</t>
+        </is>
+      </c>
+      <c r="G61" s="3" t="inlineStr">
+        <is>
+          <t>0 de 59</t>
+        </is>
+      </c>
+      <c r="H61" s="3" t="inlineStr">
+        <is>
+          <t>6 de 59</t>
+        </is>
+      </c>
+      <c r="I61" s="3" t="inlineStr">
+        <is>
+          <t>7 de 59</t>
+        </is>
+      </c>
+      <c r="J61" s="3" t="inlineStr">
+        <is>
+          <t>0 de 59</t>
+        </is>
+      </c>
+      <c r="K61" s="3" t="inlineStr">
+        <is>
+          <t>5 de 59</t>
+        </is>
+      </c>
+      <c r="L61" s="3" t="inlineStr">
+        <is>
+          <t>1 de 59</t>
+        </is>
+      </c>
+      <c r="M61" s="3" t="inlineStr">
+        <is>
+          <t>12 de 59</t>
+        </is>
+      </c>
+      <c r="N61" s="3" t="inlineStr">
+        <is>
+          <t>1 de 59</t>
+        </is>
+      </c>
+      <c r="O61" s="3" t="inlineStr">
+        <is>
+          <t>0 de 59</t>
+        </is>
+      </c>
+      <c r="P61" s="3" t="inlineStr">
+        <is>
+          <t>0 de 59</t>
+        </is>
+      </c>
+      <c r="Q61" s="3" t="inlineStr">
+        <is>
+          <t>0 de 59</t>
+        </is>
+      </c>
+      <c r="R61" s="3" t="inlineStr">
+        <is>
+          <t>0 de 59</t>
         </is>
       </c>
     </row>
@@ -4128,7 +4188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G54"/>
+  <dimension ref="A1:G55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4941,7 +5001,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>MEGGA-FRANK SAS</t>
+          <t>MARIN SANCHEZ GABRIEL ALEXANDER</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
@@ -4954,10 +5014,10 @@
         <v>0</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>6878.19</v>
+        <v>544.87</v>
       </c>
       <c r="G30" s="2" t="n">
-        <v>5000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
@@ -4968,7 +5028,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>MENA COSTA GUIDO LENNIN</t>
+          <t>MEGGA-FRANK SAS</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
@@ -4981,10 +5041,10 @@
         <v>0</v>
       </c>
       <c r="F31" s="2" t="n">
-        <v>0</v>
+        <v>6878.19</v>
       </c>
       <c r="G31" s="2" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="32">
@@ -4995,14 +5055,14 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>MENESES TORRES OSCAR LEONARDO</t>
+          <t>MENA COSTA GUIDO LENNIN</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D32" s="2" t="n">
-        <v>401.57</v>
+        <v>0</v>
       </c>
       <c r="E32" s="2" t="n">
         <v>0</v>
@@ -5011,7 +5071,7 @@
         <v>0</v>
       </c>
       <c r="G32" s="2" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33">
@@ -5022,23 +5082,23 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>MIM CONSTRUFERRETERIA E IMPORTADORA SAS</t>
+          <t>MENESES TORRES OSCAR LEONARDO</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D33" s="2" t="n">
-        <v>0</v>
+        <v>401.57</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>4583.45</v>
+        <v>0</v>
       </c>
       <c r="F33" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G33" s="2" t="n">
-        <v>2000</v>
+        <v>500</v>
       </c>
     </row>
     <row r="34">
@@ -5049,7 +5109,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>MONTAÑO JIMENEZ SANDRA GABRIELA</t>
+          <t>MIM CONSTRUFERRETERIA E IMPORTADORA SAS</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
@@ -5059,13 +5119,13 @@
         <v>0</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>1094</v>
+        <v>4583.45</v>
       </c>
       <c r="F34" s="2" t="n">
-        <v>37.75</v>
+        <v>0</v>
       </c>
       <c r="G34" s="2" t="n">
-        <v>0</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="35">
@@ -5076,20 +5136,20 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>MOROCHO BACUILIMA HILDA INES</t>
+          <t>MONTAÑO JIMENEZ SANDRA GABRIELA</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
-        <v>16.74</v>
+        <v>0</v>
       </c>
       <c r="D35" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>1133.57</v>
+        <v>1094</v>
       </c>
       <c r="F35" s="2" t="n">
-        <v>0</v>
+        <v>37.75</v>
       </c>
       <c r="G35" s="2" t="n">
         <v>0</v>
@@ -5103,17 +5163,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>MULLO GUACHO ANA LUCIA</t>
+          <t>MOROCHO BACUILIMA HILDA INES</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
-        <v>0</v>
+        <v>16.74</v>
       </c>
       <c r="D36" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E36" s="2" t="n">
-        <v>0</v>
+        <v>1133.57</v>
       </c>
       <c r="F36" s="2" t="n">
         <v>0</v>
@@ -5130,20 +5190,20 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>OCHOA OCAMPO JOHANNA SUSANA</t>
+          <t>MULLO GUACHO ANA LUCIA</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D37" s="2" t="n">
-        <v>976.9400000000001</v>
+        <v>0</v>
       </c>
       <c r="E37" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F37" s="2" t="n">
-        <v>1052.88</v>
+        <v>0</v>
       </c>
       <c r="G37" s="2" t="n">
         <v>0</v>
@@ -5157,23 +5217,23 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>PAUTA ASTUDILLO JULIO HERNAN</t>
+          <t>OCHOA OCAMPO JOHANNA SUSANA</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D38" s="2" t="n">
-        <v>321.93</v>
+        <v>976.9400000000001</v>
       </c>
       <c r="E38" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>4867.08</v>
+        <v>1052.88</v>
       </c>
       <c r="G38" s="2" t="n">
-        <v>1500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39">
@@ -5184,23 +5244,23 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>QUIÑONEZ LEON MARIA PURIFICACION</t>
+          <t>PAUTA ASTUDILLO JULIO HERNAN</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D39" s="2" t="n">
-        <v>0</v>
+        <v>321.93</v>
       </c>
       <c r="E39" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F39" s="2" t="n">
-        <v>0</v>
+        <v>4867.08</v>
       </c>
       <c r="G39" s="2" t="n">
-        <v>0</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="40">
@@ -5211,11 +5271,11 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>REYES GUILLEN VICTOR EUGENIO</t>
+          <t>QUIÑONEZ LEON MARIA PURIFICACION</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
-        <v>1882.6</v>
+        <v>0</v>
       </c>
       <c r="D40" s="2" t="n">
         <v>0</v>
@@ -5224,7 +5284,7 @@
         <v>0</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>4.06</v>
+        <v>0</v>
       </c>
       <c r="G40" s="2" t="n">
         <v>0</v>
@@ -5238,23 +5298,23 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>ROBLES CAMPOVERDE TANIA CRISTINA</t>
+          <t>REYES GUILLEN VICTOR EUGENIO</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
-        <v>101.16</v>
+        <v>1882.6</v>
       </c>
       <c r="D41" s="2" t="n">
-        <v>2180.13</v>
+        <v>0</v>
       </c>
       <c r="E41" s="2" t="n">
-        <v>3085.71</v>
+        <v>0</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>0</v>
+        <v>4.06</v>
       </c>
       <c r="G41" s="2" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42">
@@ -5265,23 +5325,23 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>ROCAFUERTE LOPEZ EVELYN ESTEFANIA</t>
+          <t>ROBLES CAMPOVERDE TANIA CRISTINA</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
-        <v>0</v>
+        <v>101.16</v>
       </c>
       <c r="D42" s="2" t="n">
-        <v>0</v>
+        <v>2180.13</v>
       </c>
       <c r="E42" s="2" t="n">
-        <v>0</v>
+        <v>3085.71</v>
       </c>
       <c r="F42" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G42" s="2" t="n">
-        <v>0</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="43">
@@ -5292,23 +5352,23 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>RUALES SARAGURO JIMMY JAVIER</t>
+          <t>ROCAFUERTE LOPEZ EVELYN ESTEFANIA</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
-        <v>9109.299999999999</v>
+        <v>0</v>
       </c>
       <c r="D43" s="2" t="n">
-        <v>5577.51</v>
+        <v>0</v>
       </c>
       <c r="E43" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F43" s="2" t="n">
-        <v>965.67</v>
+        <v>0</v>
       </c>
       <c r="G43" s="2" t="n">
-        <v>5000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44">
@@ -5319,23 +5379,23 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>SANDOVAL GONZALEZ NILO GUILLERMO</t>
+          <t>RUALES SARAGURO JIMMY JAVIER</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
-        <v>0</v>
+        <v>9109.299999999999</v>
       </c>
       <c r="D44" s="2" t="n">
-        <v>1432.86</v>
+        <v>5577.51</v>
       </c>
       <c r="E44" s="2" t="n">
-        <v>-1284.32</v>
+        <v>0</v>
       </c>
       <c r="F44" s="2" t="n">
-        <v>0</v>
+        <v>965.67</v>
       </c>
       <c r="G44" s="2" t="n">
-        <v>1200</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="45">
@@ -5346,23 +5406,23 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>SARITAMA HERRERA MARIA ELIZABETH</t>
+          <t>SANDOVAL GONZALEZ NILO GUILLERMO</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D45" s="2" t="n">
-        <v>0</v>
+        <v>1432.86</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>474.08</v>
+        <v>-1284.32</v>
       </c>
       <c r="F45" s="2" t="n">
-        <v>71.11</v>
+        <v>0</v>
       </c>
       <c r="G45" s="2" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="46">
@@ -5373,7 +5433,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>SARMIENTO SARMIENTO SANDRA EULALIA</t>
+          <t>SARITAMA HERRERA MARIA ELIZABETH</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
@@ -5383,13 +5443,13 @@
         <v>0</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>0</v>
+        <v>474.08</v>
       </c>
       <c r="F46" s="2" t="n">
-        <v>1756.19</v>
+        <v>71.11</v>
       </c>
       <c r="G46" s="2" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47">
@@ -5400,23 +5460,23 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>SIMANCAS AGUILAR HONORIO ANTONIO</t>
+          <t>SARMIENTO SARMIENTO SANDRA EULALIA</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
-        <v>3155.46</v>
+        <v>0</v>
       </c>
       <c r="D47" s="2" t="n">
-        <v>1348.76</v>
+        <v>0</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>13692.06</v>
+        <v>0</v>
       </c>
       <c r="F47" s="2" t="n">
-        <v>0</v>
+        <v>1756.19</v>
       </c>
       <c r="G47" s="2" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="48">
@@ -5427,17 +5487,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>SOPLIN MENDOZA TABITA</t>
+          <t>SIMANCAS AGUILAR HONORIO ANTONIO</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
-        <v>0</v>
+        <v>3155.46</v>
       </c>
       <c r="D48" s="2" t="n">
-        <v>0</v>
+        <v>1348.76</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>0</v>
+        <v>13692.06</v>
       </c>
       <c r="F48" s="2" t="n">
         <v>0</v>
@@ -5454,11 +5514,11 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>TAMAY SANTACRUZ MARIA ANGELICA</t>
+          <t>SOPLIN MENDOZA TABITA</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
-        <v>4237.6</v>
+        <v>0</v>
       </c>
       <c r="D49" s="2" t="n">
         <v>0</v>
@@ -5467,10 +5527,10 @@
         <v>0</v>
       </c>
       <c r="F49" s="2" t="n">
-        <v>37.75</v>
+        <v>0</v>
       </c>
       <c r="G49" s="2" t="n">
-        <v>1500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50">
@@ -5481,11 +5541,11 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
+          <t>TAMAY SANTACRUZ MARIA ANGELICA</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
-        <v>0</v>
+        <v>4237.6</v>
       </c>
       <c r="D50" s="2" t="n">
         <v>0</v>
@@ -5494,10 +5554,10 @@
         <v>0</v>
       </c>
       <c r="F50" s="2" t="n">
-        <v>0</v>
+        <v>37.75</v>
       </c>
       <c r="G50" s="2" t="n">
-        <v>2000</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="51">
@@ -5508,7 +5568,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>VEINTIMILLA JARAMILLO HERMANOS VJHNOS S.A.S.</t>
+          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
@@ -5524,7 +5584,7 @@
         <v>0</v>
       </c>
       <c r="G51" s="2" t="n">
-        <v>0</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="52">
@@ -5535,7 +5595,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>VERA CABRERA JORGE ENRIQUE</t>
+          <t>VEINTIMILLA JARAMILLO HERMANOS VJHNOS S.A.S.</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
@@ -5562,39 +5622,66 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
+          <t>VERA CABRERA JORGE ENRIQUE</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G53" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
           <t>VIVANCO MALDONADO SILVANA MARILY</t>
         </is>
       </c>
-      <c r="C53" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D53" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E53" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F53" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G53" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="C54" s="4" t="n">
+      <c r="C54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G54" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="C55" s="4" t="n">
         <v>35603.86</v>
       </c>
-      <c r="D54" s="4" t="n">
+      <c r="D55" s="4" t="n">
         <v>28143.93</v>
       </c>
-      <c r="E54" s="4" t="n">
+      <c r="E55" s="4" t="n">
         <v>43533.43</v>
       </c>
-      <c r="F54" s="4" t="n">
-        <v>42740.93</v>
-      </c>
-      <c r="G54" s="4" t="n">
+      <c r="F55" s="4" t="n">
+        <v>43285.8</v>
+      </c>
+      <c r="G55" s="4" t="n">
         <v>47200</v>
       </c>
     </row>
@@ -5787,13 +5874,13 @@
         <v>463</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>3504.7</v>
+        <v>3689.65</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>-3041.7</v>
+        <v>-3226.65</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>7.569546436285097</v>
+        <v>7.969006479481641</v>
       </c>
     </row>
     <row r="8">
@@ -5835,13 +5922,13 @@
         <v>203.76</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>2838.46</v>
+        <v>3039.78</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>-2634.7</v>
+        <v>-2836.02</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>13.93040832351786</v>
+        <v>14.91843345111896</v>
       </c>
     </row>
     <row r="10">
@@ -5859,13 +5946,13 @@
         <v>115</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>1813.8</v>
+        <v>1972.4</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>-1698.8</v>
+        <v>-1857.4</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>15.77217391304348</v>
+        <v>17.15130434782609</v>
       </c>
     </row>
     <row r="11">
@@ -5926,13 +6013,13 @@
         <v>49040.76</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>42806.72</v>
+        <v>43351.59</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>6234.039999999999</v>
+        <v>5689.169999999998</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>0.8728804366000853</v>
+        <v>0.8839909903516991</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-28 12:34:27
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R61"/>
+  <dimension ref="A1:R62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CARRION MORALES CARLOS ENRIQUE</t>
+          <t>BURNEO CELI LEYDI TATIANA</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
@@ -1137,7 +1137,7 @@
         <v>0</v>
       </c>
       <c r="M11" s="2" t="n">
-        <v>651.11</v>
+        <v>0</v>
       </c>
       <c r="N11" s="2" t="n">
         <v>0</v>
@@ -1163,7 +1163,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>COMERCIAL LUNA PAZMIÑO CIA. LTDA.</t>
+          <t>CARRION MORALES CARLOS ENRIQUE</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
@@ -1197,7 +1197,7 @@
         <v>0</v>
       </c>
       <c r="M12" s="2" t="n">
-        <v>0</v>
+        <v>651.11</v>
       </c>
       <c r="N12" s="2" t="n">
         <v>0</v>
@@ -1223,7 +1223,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>COMERCIALIZADORA RAMIREZ GALVAN CIA. LTDA</t>
+          <t>COMERCIAL LUNA PAZMIÑO CIA. LTDA.</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>CORONEL PINOS CLARA MARIA</t>
+          <t>COMERCIALIZADORA RAMIREZ GALVAN CIA. LTDA</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
@@ -1343,7 +1343,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>CORPORACION AREVALO-YUMBLA E HIJOS</t>
+          <t>CORONEL PINOS CLARA MARIA</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
@@ -1362,16 +1362,16 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>324.9</v>
+        <v>0</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>293.58</v>
+        <v>0</v>
       </c>
       <c r="J15" s="2" t="n">
         <v>0</v>
       </c>
       <c r="K15" s="2" t="n">
-        <v>213.18</v>
+        <v>0</v>
       </c>
       <c r="L15" s="2" t="n">
         <v>0</v>
@@ -1403,7 +1403,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>DIAZ CHAVEZ DIEGO FERNANDO</t>
+          <t>CORPORACION AREVALO-YUMBLA E HIJOS</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
@@ -1422,16 +1422,16 @@
         <v>0</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>0</v>
+        <v>324.9</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>0</v>
+        <v>293.58</v>
       </c>
       <c r="J16" s="2" t="n">
         <v>0</v>
       </c>
       <c r="K16" s="2" t="n">
-        <v>0</v>
+        <v>213.18</v>
       </c>
       <c r="L16" s="2" t="n">
         <v>0</v>
@@ -1463,7 +1463,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>DISTRIBUIDORA VASQUEZ ORDOÑEZ DISTRIVASOR CIA LTDA</t>
+          <t>DIAZ CHAVEZ DIEGO FERNANDO</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
@@ -1523,7 +1523,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>ESPINOZA GOMEZ LILIA ROSARIO</t>
+          <t>DISTRIBUIDORA VASQUEZ ORDOÑEZ DISTRIVASOR CIA LTDA</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
@@ -1542,16 +1542,16 @@
         <v>0</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>705.6</v>
+        <v>0</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>297.36</v>
+        <v>0</v>
       </c>
       <c r="J18" s="2" t="n">
         <v>0</v>
       </c>
       <c r="K18" s="2" t="n">
-        <v>1895.04</v>
+        <v>0</v>
       </c>
       <c r="L18" s="2" t="n">
         <v>0</v>
@@ -1583,7 +1583,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>FABIMP BENIGNO BRAVO S.A.S.</t>
+          <t>ESPINOZA GOMEZ LILIA ROSARIO</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
@@ -1602,22 +1602,22 @@
         <v>0</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>0</v>
+        <v>705.6</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>0</v>
+        <v>297.36</v>
       </c>
       <c r="J19" s="2" t="n">
         <v>0</v>
       </c>
       <c r="K19" s="2" t="n">
-        <v>0</v>
+        <v>1895.04</v>
       </c>
       <c r="L19" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M19" s="2" t="n">
-        <v>6241.39</v>
+        <v>0</v>
       </c>
       <c r="N19" s="2" t="n">
         <v>0</v>
@@ -1643,7 +1643,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>FERRICENTER EL ARENAL CIA. LTDA.</t>
+          <t>FABIMP BENIGNO BRAVO S.A.S.</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
@@ -1677,7 +1677,7 @@
         <v>0</v>
       </c>
       <c r="M20" s="2" t="n">
-        <v>0</v>
+        <v>6241.39</v>
       </c>
       <c r="N20" s="2" t="n">
         <v>0</v>
@@ -1703,7 +1703,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>FERRICRAFT S.A.S.</t>
+          <t>FERRICENTER EL ARENAL CIA. LTDA.</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
@@ -1763,7 +1763,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>FRANK FERRETERIA FRANKFERRE CIA.</t>
+          <t>FERRICRAFT S.A.S.</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
@@ -1823,7 +1823,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>GLOBAL MOYANO &amp; ASOCIADOS LEMO S.A.S.</t>
+          <t>FRANK FERRETERIA FRANKFERRE CIA.</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
@@ -1857,7 +1857,7 @@
         <v>0</v>
       </c>
       <c r="M23" s="2" t="n">
-        <v>6.32</v>
+        <v>0</v>
       </c>
       <c r="N23" s="2" t="n">
         <v>0</v>
@@ -1883,7 +1883,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>GRANDA SANDOVAL JACKELINE ELIZABETH</t>
+          <t>GLOBAL MOYANO &amp; ASOCIADOS LEMO S.A.S.</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
@@ -1917,7 +1917,7 @@
         <v>0</v>
       </c>
       <c r="M24" s="2" t="n">
-        <v>0</v>
+        <v>6.32</v>
       </c>
       <c r="N24" s="2" t="n">
         <v>0</v>
@@ -1943,7 +1943,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>HUERTA MUÑOZ NANCY ELIZABETH</t>
+          <t>GRANDA SANDOVAL JACKELINE ELIZABETH</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
@@ -2003,7 +2003,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+          <t>HUERTA MUÑOZ NANCY ELIZABETH</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
@@ -2013,7 +2013,7 @@
         <v>0</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>65.79000000000001</v>
+        <v>0</v>
       </c>
       <c r="F26" s="2" t="n">
         <v>0</v>
@@ -2063,7 +2063,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>IMPORTADORA ORTEGA CIA. LTDA.</t>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
@@ -2073,7 +2073,7 @@
         <v>0</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>0</v>
+        <v>65.79000000000001</v>
       </c>
       <c r="F27" s="2" t="n">
         <v>0</v>
@@ -2085,7 +2085,7 @@
         <v>0</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>1830.72</v>
+        <v>0</v>
       </c>
       <c r="J27" s="2" t="n">
         <v>0</v>
@@ -2097,7 +2097,7 @@
         <v>0</v>
       </c>
       <c r="M27" s="2" t="n">
-        <v>5779.47</v>
+        <v>0</v>
       </c>
       <c r="N27" s="2" t="n">
         <v>0</v>
@@ -2123,17 +2123,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>JIMBO BRITO SELENE PATRICIA</t>
+          <t>IMPORTADORA ORTEGA CIA. LTDA.</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>436.55</v>
+        <v>0</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>417.01</v>
+        <v>0</v>
       </c>
       <c r="F28" s="2" t="n">
         <v>0</v>
@@ -2142,22 +2142,22 @@
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>247.5</v>
+        <v>0</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>350.77</v>
+        <v>1830.72</v>
       </c>
       <c r="J28" s="2" t="n">
         <v>0</v>
       </c>
       <c r="K28" s="2" t="n">
-        <v>363.16</v>
+        <v>0</v>
       </c>
       <c r="L28" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M28" s="2" t="n">
-        <v>1918.73</v>
+        <v>5779.47</v>
       </c>
       <c r="N28" s="2" t="n">
         <v>0</v>
@@ -2183,17 +2183,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>JIMENEZ GORDILLO LADY KARINA</t>
+          <t>JIMBO BRITO SELENE PATRICIA</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>0</v>
+        <v>436.55</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>0</v>
+        <v>417.01</v>
       </c>
       <c r="F29" s="2" t="n">
         <v>0</v>
@@ -2202,22 +2202,22 @@
         <v>0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>0</v>
+        <v>247.5</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>0</v>
+        <v>350.77</v>
       </c>
       <c r="J29" s="2" t="n">
         <v>0</v>
       </c>
       <c r="K29" s="2" t="n">
-        <v>0</v>
+        <v>363.16</v>
       </c>
       <c r="L29" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M29" s="2" t="n">
-        <v>0</v>
+        <v>1918.73</v>
       </c>
       <c r="N29" s="2" t="n">
         <v>0</v>
@@ -2243,7 +2243,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>JUAREZ FLORES JORGE WILLIAMS</t>
+          <t>JIMENEZ GORDILLO LADY KARINA</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
@@ -2303,7 +2303,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>LEMA ESPINOZA MANUEL MARIA</t>
+          <t>JUAREZ FLORES JORGE WILLIAMS</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
@@ -2363,7 +2363,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>MARIN SANCHEZ GABRIEL ALEXANDER</t>
+          <t>LEMA ESPINOZA MANUEL MARIA</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
@@ -2385,13 +2385,13 @@
         <v>0</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>184.95</v>
+        <v>0</v>
       </c>
       <c r="J32" s="2" t="n">
         <v>0</v>
       </c>
       <c r="K32" s="2" t="n">
-        <v>201.32</v>
+        <v>0</v>
       </c>
       <c r="L32" s="2" t="n">
         <v>0</v>
@@ -2423,7 +2423,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>MEGGA-FRANK SAS</t>
+          <t>MARIN SANCHEZ GABRIEL ALEXANDER</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
@@ -2442,22 +2442,22 @@
         <v>0</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>615.6</v>
+        <v>0</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>551.99</v>
+        <v>184.95</v>
       </c>
       <c r="J33" s="2" t="n">
         <v>0</v>
       </c>
       <c r="K33" s="2" t="n">
-        <v>0</v>
+        <v>201.32</v>
       </c>
       <c r="L33" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M33" s="2" t="n">
-        <v>5710.6</v>
+        <v>0</v>
       </c>
       <c r="N33" s="2" t="n">
         <v>0</v>
@@ -2483,7 +2483,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>MENA COSTA GUIDO LENNIN</t>
+          <t>MEGGA-FRANK SAS</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
@@ -2502,10 +2502,10 @@
         <v>0</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>0</v>
+        <v>615.6</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>0</v>
+        <v>551.99</v>
       </c>
       <c r="J34" s="2" t="n">
         <v>0</v>
@@ -2517,7 +2517,7 @@
         <v>0</v>
       </c>
       <c r="M34" s="2" t="n">
-        <v>0</v>
+        <v>5710.6</v>
       </c>
       <c r="N34" s="2" t="n">
         <v>0</v>
@@ -2543,7 +2543,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>MENESES TORRES OSCAR LEONARDO</t>
+          <t>MENA COSTA GUIDO LENNIN</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
@@ -2603,7 +2603,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>MIM CONSTRUFERRETERIA E IMPORTADORA SAS</t>
+          <t>MENESES TORRES OSCAR LEONARDO</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
@@ -2663,7 +2663,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>MONTAÑO JIMENEZ SANDRA GABRIELA</t>
+          <t>MIM CONSTRUFERRETERIA E IMPORTADORA SAS</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
@@ -2723,7 +2723,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>MORALES GRACIELA ENITH</t>
+          <t>MONTAÑO JIMENEZ SANDRA GABRIELA</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>MOROCHO BACUILIMA HILDA INES</t>
+          <t>MORALES GRACIELA ENITH</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
@@ -2843,7 +2843,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>MULLO GUACHO ANA LUCIA</t>
+          <t>MOROCHO BACUILIMA HILDA INES</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
@@ -2903,7 +2903,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>OCHOA OCAMPO JOHANNA SUSANA</t>
+          <t>MULLO GUACHO ANA LUCIA</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
@@ -2931,7 +2931,7 @@
         <v>0</v>
       </c>
       <c r="K41" s="2" t="n">
-        <v>367.08</v>
+        <v>0</v>
       </c>
       <c r="L41" s="2" t="n">
         <v>0</v>
@@ -2940,7 +2940,7 @@
         <v>0</v>
       </c>
       <c r="N41" s="2" t="n">
-        <v>685.8</v>
+        <v>0</v>
       </c>
       <c r="O41" s="2" t="n">
         <v>0</v>
@@ -2963,7 +2963,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>ORTIZ GRANDA ANDREA DEL CISNE</t>
+          <t>OCHOA OCAMPO JOHANNA SUSANA</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
@@ -2991,7 +2991,7 @@
         <v>0</v>
       </c>
       <c r="K42" s="2" t="n">
-        <v>0</v>
+        <v>367.08</v>
       </c>
       <c r="L42" s="2" t="n">
         <v>0</v>
@@ -3000,7 +3000,7 @@
         <v>0</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>0</v>
+        <v>685.8</v>
       </c>
       <c r="O42" s="2" t="n">
         <v>0</v>
@@ -3023,7 +3023,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>PAUTA ASTUDILLO JULIO HERNAN</t>
+          <t>ORTIZ GRANDA ANDREA DEL CISNE</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
@@ -3057,7 +3057,7 @@
         <v>0</v>
       </c>
       <c r="M43" s="2" t="n">
-        <v>4867.08</v>
+        <v>0</v>
       </c>
       <c r="N43" s="2" t="n">
         <v>0</v>
@@ -3083,7 +3083,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>QUIÑONEZ LEON MARIA PURIFICACION</t>
+          <t>PAUTA ASTUDILLO JULIO HERNAN</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
@@ -3117,7 +3117,7 @@
         <v>0</v>
       </c>
       <c r="M44" s="2" t="n">
-        <v>0</v>
+        <v>4867.08</v>
       </c>
       <c r="N44" s="2" t="n">
         <v>0</v>
@@ -3143,7 +3143,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>REYES GUILLEN VICTOR EUGENIO</t>
+          <t>QUIÑONEZ LEON MARIA PURIFICACION</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
@@ -3203,7 +3203,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>ROBLES CAMPOVERDE TANIA CRISTINA</t>
+          <t>REYES GUILLEN VICTOR EUGENIO</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
@@ -3263,7 +3263,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>ROCAFUERTE LOPEZ EVELYN ESTEFANIA</t>
+          <t>ROBLES CAMPOVERDE TANIA CRISTINA</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
@@ -3323,7 +3323,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>RUALES SARAGURO JIMMY JAVIER</t>
+          <t>ROCAFUERTE LOPEZ EVELYN ESTEFANIA</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
@@ -3357,7 +3357,7 @@
         <v>0</v>
       </c>
       <c r="M48" s="2" t="n">
-        <v>926.02</v>
+        <v>0</v>
       </c>
       <c r="N48" s="2" t="n">
         <v>0</v>
@@ -3383,7 +3383,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>SANDOVAL GONZALEZ LAUTARO MARCELO</t>
+          <t>RUALES SARAGURO JIMMY JAVIER</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
@@ -3417,7 +3417,7 @@
         <v>0</v>
       </c>
       <c r="M49" s="2" t="n">
-        <v>0</v>
+        <v>926.02</v>
       </c>
       <c r="N49" s="2" t="n">
         <v>0</v>
@@ -3443,7 +3443,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>SANDOVAL GONZALEZ NILO GUILLERMO</t>
+          <t>SANDOVAL GONZALEZ LAUTARO MARCELO</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
@@ -3503,7 +3503,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>SANDOVAL MONTAÑO MARICELA DEL CISNE</t>
+          <t>SANDOVAL GONZALEZ NILO GUILLERMO</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
@@ -3563,7 +3563,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>SARITAMA HERRERA MARIA ELIZABETH</t>
+          <t>SANDOVAL MONTAÑO MARICELA DEL CISNE</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
@@ -3597,7 +3597,7 @@
         <v>0</v>
       </c>
       <c r="M52" s="2" t="n">
-        <v>71.11</v>
+        <v>0</v>
       </c>
       <c r="N52" s="2" t="n">
         <v>0</v>
@@ -3623,7 +3623,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>SARMIENTO SARMIENTO SANDRA EULALIA</t>
+          <t>SARITAMA HERRERA MARIA ELIZABETH</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
@@ -3633,7 +3633,7 @@
         <v>0</v>
       </c>
       <c r="E53" s="2" t="n">
-        <v>205.95</v>
+        <v>0</v>
       </c>
       <c r="F53" s="2" t="n">
         <v>0</v>
@@ -3657,7 +3657,7 @@
         <v>0</v>
       </c>
       <c r="M53" s="2" t="n">
-        <v>1550.24</v>
+        <v>71.11</v>
       </c>
       <c r="N53" s="2" t="n">
         <v>0</v>
@@ -3683,7 +3683,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>SIMANCAS AGUILAR HONORIO ANTONIO</t>
+          <t>SARMIENTO SARMIENTO SANDRA EULALIA</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
@@ -3693,7 +3693,7 @@
         <v>0</v>
       </c>
       <c r="E54" s="2" t="n">
-        <v>0</v>
+        <v>205.95</v>
       </c>
       <c r="F54" s="2" t="n">
         <v>0</v>
@@ -3717,7 +3717,7 @@
         <v>0</v>
       </c>
       <c r="M54" s="2" t="n">
-        <v>0</v>
+        <v>1550.24</v>
       </c>
       <c r="N54" s="2" t="n">
         <v>0</v>
@@ -3743,7 +3743,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>SOPLIN MENDOZA TABITA</t>
+          <t>SIMANCAS AGUILAR HONORIO ANTONIO</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
@@ -3803,7 +3803,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>TAMAY SANTACRUZ MARIA ANGELICA</t>
+          <t>SOPLIN MENDOZA TABITA</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
@@ -3863,7 +3863,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
+          <t>TAMAY SANTACRUZ MARIA ANGELICA</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
@@ -3923,7 +3923,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>VEINTIMILLA JARAMILLO HERMANOS VJHNOS S.A.S.</t>
+          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
@@ -3983,7 +3983,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>VERA CABRERA JORGE ENRIQUE</t>
+          <t>VEINTIMILLA JARAMILLO HERMANOS VJHNOS S.A.S.</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
@@ -4043,137 +4043,197 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
+          <t>VERA CABRERA JORGE ENRIQUE</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D60" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E60" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F60" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G60" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H60" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I60" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J60" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K60" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L60" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M60" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N60" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O60" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P60" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q60" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R60" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
           <t>VIVANCO MALDONADO SILVANA MARILY</t>
         </is>
       </c>
-      <c r="C60" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D60" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E60" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F60" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G60" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H60" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I60" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J60" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K60" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L60" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M60" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N60" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O60" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P60" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q60" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R60" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="C61" s="3" t="inlineStr">
-        <is>
-          <t>0 de 59</t>
-        </is>
-      </c>
-      <c r="D61" s="3" t="inlineStr">
-        <is>
-          <t>1 de 59</t>
-        </is>
-      </c>
-      <c r="E61" s="3" t="inlineStr">
-        <is>
-          <t>4 de 59</t>
-        </is>
-      </c>
-      <c r="F61" s="3" t="inlineStr">
-        <is>
-          <t>0 de 59</t>
-        </is>
-      </c>
-      <c r="G61" s="3" t="inlineStr">
-        <is>
-          <t>0 de 59</t>
-        </is>
-      </c>
-      <c r="H61" s="3" t="inlineStr">
-        <is>
-          <t>6 de 59</t>
-        </is>
-      </c>
-      <c r="I61" s="3" t="inlineStr">
-        <is>
-          <t>7 de 59</t>
-        </is>
-      </c>
-      <c r="J61" s="3" t="inlineStr">
-        <is>
-          <t>0 de 59</t>
-        </is>
-      </c>
-      <c r="K61" s="3" t="inlineStr">
-        <is>
-          <t>5 de 59</t>
-        </is>
-      </c>
-      <c r="L61" s="3" t="inlineStr">
-        <is>
-          <t>1 de 59</t>
-        </is>
-      </c>
-      <c r="M61" s="3" t="inlineStr">
-        <is>
-          <t>13 de 59</t>
-        </is>
-      </c>
-      <c r="N61" s="3" t="inlineStr">
-        <is>
-          <t>1 de 59</t>
-        </is>
-      </c>
-      <c r="O61" s="3" t="inlineStr">
-        <is>
-          <t>0 de 59</t>
-        </is>
-      </c>
-      <c r="P61" s="3" t="inlineStr">
-        <is>
-          <t>0 de 59</t>
-        </is>
-      </c>
-      <c r="Q61" s="3" t="inlineStr">
-        <is>
-          <t>0 de 59</t>
-        </is>
-      </c>
-      <c r="R61" s="3" t="inlineStr">
-        <is>
-          <t>0 de 59</t>
+      <c r="C61" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D61" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E61" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F61" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G61" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H61" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I61" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J61" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K61" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L61" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M61" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N61" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O61" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P61" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q61" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R61" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>0 de 60</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>1 de 60</t>
+        </is>
+      </c>
+      <c r="E62" s="3" t="inlineStr">
+        <is>
+          <t>4 de 60</t>
+        </is>
+      </c>
+      <c r="F62" s="3" t="inlineStr">
+        <is>
+          <t>0 de 60</t>
+        </is>
+      </c>
+      <c r="G62" s="3" t="inlineStr">
+        <is>
+          <t>0 de 60</t>
+        </is>
+      </c>
+      <c r="H62" s="3" t="inlineStr">
+        <is>
+          <t>6 de 60</t>
+        </is>
+      </c>
+      <c r="I62" s="3" t="inlineStr">
+        <is>
+          <t>7 de 60</t>
+        </is>
+      </c>
+      <c r="J62" s="3" t="inlineStr">
+        <is>
+          <t>0 de 60</t>
+        </is>
+      </c>
+      <c r="K62" s="3" t="inlineStr">
+        <is>
+          <t>5 de 60</t>
+        </is>
+      </c>
+      <c r="L62" s="3" t="inlineStr">
+        <is>
+          <t>1 de 60</t>
+        </is>
+      </c>
+      <c r="M62" s="3" t="inlineStr">
+        <is>
+          <t>13 de 60</t>
+        </is>
+      </c>
+      <c r="N62" s="3" t="inlineStr">
+        <is>
+          <t>1 de 60</t>
+        </is>
+      </c>
+      <c r="O62" s="3" t="inlineStr">
+        <is>
+          <t>0 de 60</t>
+        </is>
+      </c>
+      <c r="P62" s="3" t="inlineStr">
+        <is>
+          <t>0 de 60</t>
+        </is>
+      </c>
+      <c r="Q62" s="3" t="inlineStr">
+        <is>
+          <t>0 de 60</t>
+        </is>
+      </c>
+      <c r="R62" s="3" t="inlineStr">
+        <is>
+          <t>0 de 60</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4248,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G55"/>
+  <dimension ref="A1:G56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4542,23 +4602,23 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>CARRION MORALES CARLOS ENRIQUE</t>
+          <t>BURNEO CELI LEYDI TATIANA</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>50.54</v>
+        <v>0</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>258.49</v>
+        <v>0</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>651.11</v>
+        <v>0</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -4569,23 +4629,23 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>COMERCIAL LUNA PAZMIÑO CIA. LTDA.</t>
+          <t>CARRION MORALES CARLOS ENRIQUE</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>0</v>
+        <v>50.54</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>0</v>
+        <v>258.49</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>0</v>
+        <v>651.11</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>0</v>
+        <v>500</v>
       </c>
     </row>
     <row r="15">
@@ -4596,23 +4656,23 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>CORONEL PINOS CLARA MARIA</t>
+          <t>COMERCIAL LUNA PAZMIÑO CIA. LTDA.</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>2068.01</v>
+        <v>0</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>5446.06</v>
+        <v>0</v>
       </c>
       <c r="F15" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>1500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -4623,20 +4683,20 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>CORPORACION AREVALO-YUMBLA E HIJOS</t>
+          <t>CORONEL PINOS CLARA MARIA</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>0</v>
+        <v>2068.01</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>0</v>
+        <v>5446.06</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>1214.7</v>
+        <v>0</v>
       </c>
       <c r="G16" s="2" t="n">
         <v>1500</v>
@@ -4650,7 +4710,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>DIAZ CHAVEZ DIEGO FERNANDO</t>
+          <t>CORPORACION AREVALO-YUMBLA E HIJOS</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
@@ -4663,10 +4723,10 @@
         <v>0</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>0</v>
+        <v>1214.7</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>0</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="18">
@@ -4677,7 +4737,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>DISTRIBUIDORA VASQUEZ ORDOÑEZ DISTRIVASOR CIA LTDA</t>
+          <t>DIAZ CHAVEZ DIEGO FERNANDO</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
@@ -4693,7 +4753,7 @@
         <v>0</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -4704,23 +4764,23 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ESPINOZA GOMEZ LILIA ROSARIO</t>
+          <t>DISTRIBUIDORA VASQUEZ ORDOÑEZ DISTRIVASOR CIA LTDA</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>3072.2</v>
+        <v>0</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>426.67</v>
+        <v>0</v>
       </c>
       <c r="E19" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>2898</v>
+        <v>0</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>3000</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="20">
@@ -4731,23 +4791,23 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>FABIMP BENIGNO BRAVO S.A.S.</t>
+          <t>ESPINOZA GOMEZ LILIA ROSARIO</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>0</v>
+        <v>3072.2</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>3603.22</v>
+        <v>426.67</v>
       </c>
       <c r="E20" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>6241.39</v>
+        <v>2898</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>2000</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="21">
@@ -4758,23 +4818,23 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>FERRICENTER EL ARENAL CIA. LTDA.</t>
+          <t>FABIMP BENIGNO BRAVO S.A.S.</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>4096.36</v>
+        <v>0</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>0</v>
+        <v>3603.22</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>1550.24</v>
+        <v>0</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>0</v>
+        <v>6241.39</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>1500</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="22">
@@ -4785,23 +4845,23 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>GLOBAL MOYANO &amp; ASOCIADOS LEMO S.A.S.</t>
+          <t>FERRICENTER EL ARENAL CIA. LTDA.</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>70.37</v>
+        <v>4096.36</v>
       </c>
       <c r="D22" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>0</v>
+        <v>1550.24</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>19.66</v>
+        <v>0</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>0</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="23">
@@ -4812,20 +4872,20 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>GRANDA SANDOVAL JACKELINE ELIZABETH</t>
+          <t>GLOBAL MOYANO &amp; ASOCIADOS LEMO S.A.S.</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>0</v>
+        <v>70.37</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>1045.76</v>
+        <v>0</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>68.23</v>
+        <v>0</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>0</v>
+        <v>19.66</v>
       </c>
       <c r="G23" s="2" t="n">
         <v>0</v>
@@ -4839,23 +4899,23 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>HUERTA MUÑOZ NANCY ELIZABETH</t>
+          <t>GRANDA SANDOVAL JACKELINE ELIZABETH</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>4922.83</v>
+        <v>0</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>0</v>
+        <v>1045.76</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>1499.16</v>
+        <v>68.23</v>
       </c>
       <c r="F24" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -4866,23 +4926,23 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>IMPORTADORA ORTEGA CIA. LTDA.</t>
+          <t>HUERTA MUÑOZ NANCY ELIZABETH</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>0</v>
+        <v>4922.83</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>1479.64</v>
+        <v>0</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>11932.7</v>
+        <v>1499.16</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>7610.19</v>
+        <v>0</v>
       </c>
       <c r="G25" s="2" t="n">
-        <v>4000</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="26">
@@ -4893,23 +4953,23 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>JIMBO BRITO SELENE PATRICIA</t>
+          <t>IMPORTADORA ORTEGA CIA. LTDA.</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>0</v>
+        <v>1479.64</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>0</v>
+        <v>11932.7</v>
       </c>
       <c r="F26" s="2" t="n">
-        <v>5097.28</v>
+        <v>7610.19</v>
       </c>
       <c r="G26" s="2" t="n">
-        <v>0</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="27">
@@ -4920,7 +4980,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>JIMENEZ GORDILLO LADY KARINA</t>
+          <t>JIMBO BRITO SELENE PATRICIA</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
@@ -4933,7 +4993,7 @@
         <v>0</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>0</v>
+        <v>5097.28</v>
       </c>
       <c r="G27" s="2" t="n">
         <v>0</v>
@@ -4947,7 +5007,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>JUAREZ FLORES JORGE WILLIAMS</t>
+          <t>JIMENEZ GORDILLO LADY KARINA</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
@@ -4974,11 +5034,11 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>LEMA ESPINOZA MANUEL MARIA</t>
+          <t>JUAREZ FLORES JORGE WILLIAMS</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>865.47</v>
+        <v>0</v>
       </c>
       <c r="D29" s="2" t="n">
         <v>0</v>
@@ -4990,7 +5050,7 @@
         <v>0</v>
       </c>
       <c r="G29" s="2" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
@@ -5001,11 +5061,11 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>MARIN SANCHEZ GABRIEL ALEXANDER</t>
+          <t>LEMA ESPINOZA MANUEL MARIA</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>0</v>
+        <v>865.47</v>
       </c>
       <c r="D30" s="2" t="n">
         <v>0</v>
@@ -5014,10 +5074,10 @@
         <v>0</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>544.87</v>
+        <v>0</v>
       </c>
       <c r="G30" s="2" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="31">
@@ -5028,7 +5088,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>MEGGA-FRANK SAS</t>
+          <t>MARIN SANCHEZ GABRIEL ALEXANDER</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
@@ -5041,10 +5101,10 @@
         <v>0</v>
       </c>
       <c r="F31" s="2" t="n">
-        <v>6878.19</v>
+        <v>544.87</v>
       </c>
       <c r="G31" s="2" t="n">
-        <v>5000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
@@ -5055,7 +5115,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>MENA COSTA GUIDO LENNIN</t>
+          <t>MEGGA-FRANK SAS</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
@@ -5068,10 +5128,10 @@
         <v>0</v>
       </c>
       <c r="F32" s="2" t="n">
-        <v>0</v>
+        <v>6878.19</v>
       </c>
       <c r="G32" s="2" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="33">
@@ -5082,14 +5142,14 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>MENESES TORRES OSCAR LEONARDO</t>
+          <t>MENA COSTA GUIDO LENNIN</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D33" s="2" t="n">
-        <v>401.57</v>
+        <v>0</v>
       </c>
       <c r="E33" s="2" t="n">
         <v>0</v>
@@ -5098,7 +5158,7 @@
         <v>0</v>
       </c>
       <c r="G33" s="2" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34">
@@ -5109,23 +5169,23 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>MIM CONSTRUFERRETERIA E IMPORTADORA SAS</t>
+          <t>MENESES TORRES OSCAR LEONARDO</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D34" s="2" t="n">
-        <v>0</v>
+        <v>401.57</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>4583.45</v>
+        <v>0</v>
       </c>
       <c r="F34" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G34" s="2" t="n">
-        <v>2000</v>
+        <v>500</v>
       </c>
     </row>
     <row r="35">
@@ -5136,7 +5196,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>MONTAÑO JIMENEZ SANDRA GABRIELA</t>
+          <t>MIM CONSTRUFERRETERIA E IMPORTADORA SAS</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
@@ -5146,13 +5206,13 @@
         <v>0</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>1094</v>
+        <v>4583.45</v>
       </c>
       <c r="F35" s="2" t="n">
-        <v>37.75</v>
+        <v>0</v>
       </c>
       <c r="G35" s="2" t="n">
-        <v>0</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="36">
@@ -5163,20 +5223,20 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>MOROCHO BACUILIMA HILDA INES</t>
+          <t>MONTAÑO JIMENEZ SANDRA GABRIELA</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
-        <v>16.74</v>
+        <v>0</v>
       </c>
       <c r="D36" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E36" s="2" t="n">
-        <v>1133.57</v>
+        <v>1094</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>0</v>
+        <v>37.75</v>
       </c>
       <c r="G36" s="2" t="n">
         <v>0</v>
@@ -5190,17 +5250,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>MULLO GUACHO ANA LUCIA</t>
+          <t>MOROCHO BACUILIMA HILDA INES</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
-        <v>0</v>
+        <v>16.74</v>
       </c>
       <c r="D37" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>0</v>
+        <v>1133.57</v>
       </c>
       <c r="F37" s="2" t="n">
         <v>0</v>
@@ -5217,20 +5277,20 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>OCHOA OCAMPO JOHANNA SUSANA</t>
+          <t>MULLO GUACHO ANA LUCIA</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D38" s="2" t="n">
-        <v>976.9400000000001</v>
+        <v>0</v>
       </c>
       <c r="E38" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>1052.88</v>
+        <v>0</v>
       </c>
       <c r="G38" s="2" t="n">
         <v>0</v>
@@ -5244,23 +5304,23 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>PAUTA ASTUDILLO JULIO HERNAN</t>
+          <t>OCHOA OCAMPO JOHANNA SUSANA</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D39" s="2" t="n">
-        <v>321.93</v>
+        <v>976.9400000000001</v>
       </c>
       <c r="E39" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F39" s="2" t="n">
-        <v>4867.08</v>
+        <v>1052.88</v>
       </c>
       <c r="G39" s="2" t="n">
-        <v>1500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40">
@@ -5271,23 +5331,23 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>QUIÑONEZ LEON MARIA PURIFICACION</t>
+          <t>PAUTA ASTUDILLO JULIO HERNAN</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D40" s="2" t="n">
-        <v>0</v>
+        <v>321.93</v>
       </c>
       <c r="E40" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>0</v>
+        <v>4867.08</v>
       </c>
       <c r="G40" s="2" t="n">
-        <v>0</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="41">
@@ -5298,11 +5358,11 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>REYES GUILLEN VICTOR EUGENIO</t>
+          <t>QUIÑONEZ LEON MARIA PURIFICACION</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
-        <v>1882.6</v>
+        <v>0</v>
       </c>
       <c r="D41" s="2" t="n">
         <v>0</v>
@@ -5311,7 +5371,7 @@
         <v>0</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>4.06</v>
+        <v>0</v>
       </c>
       <c r="G41" s="2" t="n">
         <v>0</v>
@@ -5325,23 +5385,23 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>ROBLES CAMPOVERDE TANIA CRISTINA</t>
+          <t>REYES GUILLEN VICTOR EUGENIO</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
-        <v>101.16</v>
+        <v>1882.6</v>
       </c>
       <c r="D42" s="2" t="n">
-        <v>2180.13</v>
+        <v>0</v>
       </c>
       <c r="E42" s="2" t="n">
-        <v>3085.71</v>
+        <v>0</v>
       </c>
       <c r="F42" s="2" t="n">
-        <v>0</v>
+        <v>4.06</v>
       </c>
       <c r="G42" s="2" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43">
@@ -5352,23 +5412,23 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>ROCAFUERTE LOPEZ EVELYN ESTEFANIA</t>
+          <t>ROBLES CAMPOVERDE TANIA CRISTINA</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
-        <v>0</v>
+        <v>101.16</v>
       </c>
       <c r="D43" s="2" t="n">
-        <v>0</v>
+        <v>2180.13</v>
       </c>
       <c r="E43" s="2" t="n">
-        <v>0</v>
+        <v>3085.71</v>
       </c>
       <c r="F43" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G43" s="2" t="n">
-        <v>0</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="44">
@@ -5379,23 +5439,23 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>RUALES SARAGURO JIMMY JAVIER</t>
+          <t>ROCAFUERTE LOPEZ EVELYN ESTEFANIA</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
-        <v>9109.299999999999</v>
+        <v>0</v>
       </c>
       <c r="D44" s="2" t="n">
-        <v>5577.51</v>
+        <v>0</v>
       </c>
       <c r="E44" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F44" s="2" t="n">
-        <v>965.67</v>
+        <v>0</v>
       </c>
       <c r="G44" s="2" t="n">
-        <v>5000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45">
@@ -5406,23 +5466,23 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>SANDOVAL GONZALEZ NILO GUILLERMO</t>
+          <t>RUALES SARAGURO JIMMY JAVIER</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
-        <v>0</v>
+        <v>9109.299999999999</v>
       </c>
       <c r="D45" s="2" t="n">
-        <v>1432.86</v>
+        <v>5577.51</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>-1284.32</v>
+        <v>0</v>
       </c>
       <c r="F45" s="2" t="n">
-        <v>0</v>
+        <v>965.67</v>
       </c>
       <c r="G45" s="2" t="n">
-        <v>1200</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="46">
@@ -5433,23 +5493,23 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>SARITAMA HERRERA MARIA ELIZABETH</t>
+          <t>SANDOVAL GONZALEZ NILO GUILLERMO</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D46" s="2" t="n">
-        <v>0</v>
+        <v>1432.86</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>474.08</v>
+        <v>-1284.32</v>
       </c>
       <c r="F46" s="2" t="n">
-        <v>71.11</v>
+        <v>0</v>
       </c>
       <c r="G46" s="2" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="47">
@@ -5460,7 +5520,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>SARMIENTO SARMIENTO SANDRA EULALIA</t>
+          <t>SARITAMA HERRERA MARIA ELIZABETH</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
@@ -5470,13 +5530,13 @@
         <v>0</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>0</v>
+        <v>474.08</v>
       </c>
       <c r="F47" s="2" t="n">
-        <v>1756.19</v>
+        <v>71.11</v>
       </c>
       <c r="G47" s="2" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48">
@@ -5487,23 +5547,23 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>SIMANCAS AGUILAR HONORIO ANTONIO</t>
+          <t>SARMIENTO SARMIENTO SANDRA EULALIA</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
-        <v>3155.46</v>
+        <v>0</v>
       </c>
       <c r="D48" s="2" t="n">
-        <v>1348.76</v>
+        <v>0</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>13692.06</v>
+        <v>0</v>
       </c>
       <c r="F48" s="2" t="n">
-        <v>0</v>
+        <v>1756.19</v>
       </c>
       <c r="G48" s="2" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="49">
@@ -5514,17 +5574,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>SOPLIN MENDOZA TABITA</t>
+          <t>SIMANCAS AGUILAR HONORIO ANTONIO</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
-        <v>0</v>
+        <v>3155.46</v>
       </c>
       <c r="D49" s="2" t="n">
-        <v>0</v>
+        <v>1348.76</v>
       </c>
       <c r="E49" s="2" t="n">
-        <v>0</v>
+        <v>13692.06</v>
       </c>
       <c r="F49" s="2" t="n">
         <v>0</v>
@@ -5541,11 +5601,11 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>TAMAY SANTACRUZ MARIA ANGELICA</t>
+          <t>SOPLIN MENDOZA TABITA</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
-        <v>4237.6</v>
+        <v>0</v>
       </c>
       <c r="D50" s="2" t="n">
         <v>0</v>
@@ -5554,10 +5614,10 @@
         <v>0</v>
       </c>
       <c r="F50" s="2" t="n">
-        <v>37.75</v>
+        <v>0</v>
       </c>
       <c r="G50" s="2" t="n">
-        <v>1500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="51">
@@ -5568,11 +5628,11 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
+          <t>TAMAY SANTACRUZ MARIA ANGELICA</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
-        <v>0</v>
+        <v>4237.6</v>
       </c>
       <c r="D51" s="2" t="n">
         <v>0</v>
@@ -5581,10 +5641,10 @@
         <v>0</v>
       </c>
       <c r="F51" s="2" t="n">
-        <v>0</v>
+        <v>37.75</v>
       </c>
       <c r="G51" s="2" t="n">
-        <v>2000</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="52">
@@ -5595,7 +5655,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>VEINTIMILLA JARAMILLO HERMANOS VJHNOS S.A.S.</t>
+          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
@@ -5611,7 +5671,7 @@
         <v>0</v>
       </c>
       <c r="G52" s="2" t="n">
-        <v>0</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="53">
@@ -5622,7 +5682,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>VERA CABRERA JORGE ENRIQUE</t>
+          <t>VEINTIMILLA JARAMILLO HERMANOS VJHNOS S.A.S.</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
@@ -5649,39 +5709,66 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
+          <t>VERA CABRERA JORGE ENRIQUE</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G54" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
           <t>VIVANCO MALDONADO SILVANA MARILY</t>
         </is>
       </c>
-      <c r="C54" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D54" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E54" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F54" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G54" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="C55" s="4" t="n">
+      <c r="C55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G55" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="C56" s="4" t="n">
         <v>35603.86</v>
       </c>
-      <c r="D55" s="4" t="n">
+      <c r="D56" s="4" t="n">
         <v>28143.93</v>
       </c>
-      <c r="E55" s="4" t="n">
+      <c r="E56" s="4" t="n">
         <v>43533.43</v>
       </c>
-      <c r="F55" s="4" t="n">
+      <c r="F56" s="4" t="n">
         <v>43936.91</v>
       </c>
-      <c r="G55" s="4" t="n">
+      <c r="G56" s="4" t="n">
         <v>47200</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática 2026-09-28 12:42:29
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R62"/>
+  <dimension ref="A1:R59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2543,7 +2543,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>MENA COSTA GUIDO LENNIN</t>
+          <t>MENESES TORRES OSCAR LEONARDO</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
@@ -2603,7 +2603,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>MENESES TORRES OSCAR LEONARDO</t>
+          <t>MIM CONSTRUFERRETERIA E IMPORTADORA SAS</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
@@ -2663,7 +2663,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>MIM CONSTRUFERRETERIA E IMPORTADORA SAS</t>
+          <t>MONTAÑO JIMENEZ SANDRA GABRIELA</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
@@ -2723,7 +2723,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>MONTAÑO JIMENEZ SANDRA GABRIELA</t>
+          <t>MORALES GRACIELA ENITH</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>MORALES GRACIELA ENITH</t>
+          <t>MOROCHO BACUILIMA HILDA INES</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
@@ -2843,7 +2843,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>MOROCHO BACUILIMA HILDA INES</t>
+          <t>MULLO GUACHO ANA LUCIA</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
@@ -2903,7 +2903,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>MULLO GUACHO ANA LUCIA</t>
+          <t>OCHOA OCAMPO JOHANNA SUSANA</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
@@ -2931,7 +2931,7 @@
         <v>0</v>
       </c>
       <c r="K41" s="2" t="n">
-        <v>0</v>
+        <v>367.08</v>
       </c>
       <c r="L41" s="2" t="n">
         <v>0</v>
@@ -2940,7 +2940,7 @@
         <v>0</v>
       </c>
       <c r="N41" s="2" t="n">
-        <v>0</v>
+        <v>685.8</v>
       </c>
       <c r="O41" s="2" t="n">
         <v>0</v>
@@ -2963,7 +2963,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>OCHOA OCAMPO JOHANNA SUSANA</t>
+          <t>ORTIZ GRANDA ANDREA DEL CISNE</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
@@ -2991,7 +2991,7 @@
         <v>0</v>
       </c>
       <c r="K42" s="2" t="n">
-        <v>367.08</v>
+        <v>0</v>
       </c>
       <c r="L42" s="2" t="n">
         <v>0</v>
@@ -3000,7 +3000,7 @@
         <v>0</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>685.8</v>
+        <v>0</v>
       </c>
       <c r="O42" s="2" t="n">
         <v>0</v>
@@ -3023,7 +3023,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>ORTIZ GRANDA ANDREA DEL CISNE</t>
+          <t>PAUTA ASTUDILLO JULIO HERNAN</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
@@ -3057,7 +3057,7 @@
         <v>0</v>
       </c>
       <c r="M43" s="2" t="n">
-        <v>0</v>
+        <v>4867.08</v>
       </c>
       <c r="N43" s="2" t="n">
         <v>0</v>
@@ -3083,7 +3083,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>PAUTA ASTUDILLO JULIO HERNAN</t>
+          <t>REYES GUILLEN VICTOR EUGENIO</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
@@ -3117,7 +3117,7 @@
         <v>0</v>
       </c>
       <c r="M44" s="2" t="n">
-        <v>4867.08</v>
+        <v>0</v>
       </c>
       <c r="N44" s="2" t="n">
         <v>0</v>
@@ -3143,7 +3143,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>QUIÑONEZ LEON MARIA PURIFICACION</t>
+          <t>ROBLES CAMPOVERDE TANIA CRISTINA</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
@@ -3203,7 +3203,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>REYES GUILLEN VICTOR EUGENIO</t>
+          <t>ROCAFUERTE LOPEZ EVELYN ESTEFANIA</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
@@ -3263,7 +3263,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>ROBLES CAMPOVERDE TANIA CRISTINA</t>
+          <t>RUALES SARAGURO JIMMY JAVIER</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
@@ -3297,7 +3297,7 @@
         <v>0</v>
       </c>
       <c r="M47" s="2" t="n">
-        <v>0</v>
+        <v>926.02</v>
       </c>
       <c r="N47" s="2" t="n">
         <v>0</v>
@@ -3323,7 +3323,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>ROCAFUERTE LOPEZ EVELYN ESTEFANIA</t>
+          <t>SANDOVAL GONZALEZ LAUTARO MARCELO</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
@@ -3383,7 +3383,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>RUALES SARAGURO JIMMY JAVIER</t>
+          <t>SANDOVAL GONZALEZ NILO GUILLERMO</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
@@ -3417,7 +3417,7 @@
         <v>0</v>
       </c>
       <c r="M49" s="2" t="n">
-        <v>926.02</v>
+        <v>0</v>
       </c>
       <c r="N49" s="2" t="n">
         <v>0</v>
@@ -3443,7 +3443,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>SANDOVAL GONZALEZ LAUTARO MARCELO</t>
+          <t>SANDOVAL MONTAÑO MARICELA DEL CISNE</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
@@ -3503,7 +3503,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>SANDOVAL GONZALEZ NILO GUILLERMO</t>
+          <t>SARITAMA HERRERA MARIA ELIZABETH</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
@@ -3537,7 +3537,7 @@
         <v>0</v>
       </c>
       <c r="M51" s="2" t="n">
-        <v>0</v>
+        <v>71.11</v>
       </c>
       <c r="N51" s="2" t="n">
         <v>0</v>
@@ -3563,7 +3563,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>SANDOVAL MONTAÑO MARICELA DEL CISNE</t>
+          <t>SARMIENTO SARMIENTO SANDRA EULALIA</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
@@ -3573,7 +3573,7 @@
         <v>0</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>0</v>
+        <v>205.95</v>
       </c>
       <c r="F52" s="2" t="n">
         <v>0</v>
@@ -3597,7 +3597,7 @@
         <v>0</v>
       </c>
       <c r="M52" s="2" t="n">
-        <v>0</v>
+        <v>1550.24</v>
       </c>
       <c r="N52" s="2" t="n">
         <v>0</v>
@@ -3623,7 +3623,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>SARITAMA HERRERA MARIA ELIZABETH</t>
+          <t>SIMANCAS AGUILAR HONORIO ANTONIO</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
@@ -3657,7 +3657,7 @@
         <v>0</v>
       </c>
       <c r="M53" s="2" t="n">
-        <v>71.11</v>
+        <v>0</v>
       </c>
       <c r="N53" s="2" t="n">
         <v>0</v>
@@ -3683,7 +3683,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>SARMIENTO SARMIENTO SANDRA EULALIA</t>
+          <t>TAMAY SANTACRUZ MARIA ANGELICA</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
@@ -3693,7 +3693,7 @@
         <v>0</v>
       </c>
       <c r="E54" s="2" t="n">
-        <v>205.95</v>
+        <v>0</v>
       </c>
       <c r="F54" s="2" t="n">
         <v>0</v>
@@ -3717,7 +3717,7 @@
         <v>0</v>
       </c>
       <c r="M54" s="2" t="n">
-        <v>1550.24</v>
+        <v>0</v>
       </c>
       <c r="N54" s="2" t="n">
         <v>0</v>
@@ -3743,7 +3743,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>SIMANCAS AGUILAR HONORIO ANTONIO</t>
+          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
@@ -3803,7 +3803,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>SOPLIN MENDOZA TABITA</t>
+          <t>VEINTIMILLA JARAMILLO HERMANOS VJHNOS S.A.S.</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
@@ -3863,7 +3863,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>TAMAY SANTACRUZ MARIA ANGELICA</t>
+          <t>VERA CABRERA JORGE ENRIQUE</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
@@ -3923,7 +3923,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
+          <t>VIVANCO MALDONADO SILVANA MARILY</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
@@ -3976,264 +3976,84 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>VEINTIMILLA JARAMILLO HERMANOS VJHNOS S.A.S.</t>
-        </is>
-      </c>
-      <c r="C59" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D59" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E59" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F59" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G59" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H59" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I59" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J59" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K59" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L59" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M59" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N59" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O59" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P59" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q59" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R59" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>VERA CABRERA JORGE ENRIQUE</t>
-        </is>
-      </c>
-      <c r="C60" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D60" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E60" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F60" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G60" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H60" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I60" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J60" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K60" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L60" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M60" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N60" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O60" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P60" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q60" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R60" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>VIVANCO MALDONADO SILVANA MARILY</t>
-        </is>
-      </c>
-      <c r="C61" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D61" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E61" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F61" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G61" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H61" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I61" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J61" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K61" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L61" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M61" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N61" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O61" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P61" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q61" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R61" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="C62" s="3" t="inlineStr">
-        <is>
-          <t>0 de 60</t>
-        </is>
-      </c>
-      <c r="D62" s="3" t="inlineStr">
-        <is>
-          <t>1 de 60</t>
-        </is>
-      </c>
-      <c r="E62" s="3" t="inlineStr">
-        <is>
-          <t>4 de 60</t>
-        </is>
-      </c>
-      <c r="F62" s="3" t="inlineStr">
-        <is>
-          <t>0 de 60</t>
-        </is>
-      </c>
-      <c r="G62" s="3" t="inlineStr">
-        <is>
-          <t>0 de 60</t>
-        </is>
-      </c>
-      <c r="H62" s="3" t="inlineStr">
-        <is>
-          <t>6 de 60</t>
-        </is>
-      </c>
-      <c r="I62" s="3" t="inlineStr">
-        <is>
-          <t>7 de 60</t>
-        </is>
-      </c>
-      <c r="J62" s="3" t="inlineStr">
-        <is>
-          <t>0 de 60</t>
-        </is>
-      </c>
-      <c r="K62" s="3" t="inlineStr">
-        <is>
-          <t>5 de 60</t>
-        </is>
-      </c>
-      <c r="L62" s="3" t="inlineStr">
-        <is>
-          <t>1 de 60</t>
-        </is>
-      </c>
-      <c r="M62" s="3" t="inlineStr">
-        <is>
-          <t>13 de 60</t>
-        </is>
-      </c>
-      <c r="N62" s="3" t="inlineStr">
-        <is>
-          <t>1 de 60</t>
-        </is>
-      </c>
-      <c r="O62" s="3" t="inlineStr">
-        <is>
-          <t>0 de 60</t>
-        </is>
-      </c>
-      <c r="P62" s="3" t="inlineStr">
-        <is>
-          <t>0 de 60</t>
-        </is>
-      </c>
-      <c r="Q62" s="3" t="inlineStr">
-        <is>
-          <t>0 de 60</t>
-        </is>
-      </c>
-      <c r="R62" s="3" t="inlineStr">
-        <is>
-          <t>0 de 60</t>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>0 de 57</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t>1 de 57</t>
+        </is>
+      </c>
+      <c r="E59" s="3" t="inlineStr">
+        <is>
+          <t>4 de 57</t>
+        </is>
+      </c>
+      <c r="F59" s="3" t="inlineStr">
+        <is>
+          <t>0 de 57</t>
+        </is>
+      </c>
+      <c r="G59" s="3" t="inlineStr">
+        <is>
+          <t>0 de 57</t>
+        </is>
+      </c>
+      <c r="H59" s="3" t="inlineStr">
+        <is>
+          <t>6 de 57</t>
+        </is>
+      </c>
+      <c r="I59" s="3" t="inlineStr">
+        <is>
+          <t>7 de 57</t>
+        </is>
+      </c>
+      <c r="J59" s="3" t="inlineStr">
+        <is>
+          <t>0 de 57</t>
+        </is>
+      </c>
+      <c r="K59" s="3" t="inlineStr">
+        <is>
+          <t>5 de 57</t>
+        </is>
+      </c>
+      <c r="L59" s="3" t="inlineStr">
+        <is>
+          <t>1 de 57</t>
+        </is>
+      </c>
+      <c r="M59" s="3" t="inlineStr">
+        <is>
+          <t>13 de 57</t>
+        </is>
+      </c>
+      <c r="N59" s="3" t="inlineStr">
+        <is>
+          <t>1 de 57</t>
+        </is>
+      </c>
+      <c r="O59" s="3" t="inlineStr">
+        <is>
+          <t>0 de 57</t>
+        </is>
+      </c>
+      <c r="P59" s="3" t="inlineStr">
+        <is>
+          <t>0 de 57</t>
+        </is>
+      </c>
+      <c r="Q59" s="3" t="inlineStr">
+        <is>
+          <t>0 de 57</t>
+        </is>
+      </c>
+      <c r="R59" s="3" t="inlineStr">
+        <is>
+          <t>0 de 57</t>
         </is>
       </c>
     </row>
@@ -4248,7 +4068,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G56"/>
+  <dimension ref="A1:G53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -5142,14 +4962,14 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>MENA COSTA GUIDO LENNIN</t>
+          <t>MENESES TORRES OSCAR LEONARDO</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D33" s="2" t="n">
-        <v>0</v>
+        <v>401.57</v>
       </c>
       <c r="E33" s="2" t="n">
         <v>0</v>
@@ -5158,7 +4978,7 @@
         <v>0</v>
       </c>
       <c r="G33" s="2" t="n">
-        <v>0</v>
+        <v>500</v>
       </c>
     </row>
     <row r="34">
@@ -5169,23 +4989,23 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>MENESES TORRES OSCAR LEONARDO</t>
+          <t>MIM CONSTRUFERRETERIA E IMPORTADORA SAS</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D34" s="2" t="n">
-        <v>401.57</v>
+        <v>0</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>0</v>
+        <v>4583.45</v>
       </c>
       <c r="F34" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G34" s="2" t="n">
-        <v>500</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="35">
@@ -5196,7 +5016,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>MIM CONSTRUFERRETERIA E IMPORTADORA SAS</t>
+          <t>MONTAÑO JIMENEZ SANDRA GABRIELA</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
@@ -5206,13 +5026,13 @@
         <v>0</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>4583.45</v>
+        <v>1094</v>
       </c>
       <c r="F35" s="2" t="n">
-        <v>0</v>
+        <v>37.75</v>
       </c>
       <c r="G35" s="2" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
@@ -5223,20 +5043,20 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>MONTAÑO JIMENEZ SANDRA GABRIELA</t>
+          <t>MOROCHO BACUILIMA HILDA INES</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
-        <v>0</v>
+        <v>16.74</v>
       </c>
       <c r="D36" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E36" s="2" t="n">
-        <v>1094</v>
+        <v>1133.57</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>37.75</v>
+        <v>0</v>
       </c>
       <c r="G36" s="2" t="n">
         <v>0</v>
@@ -5250,17 +5070,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>MOROCHO BACUILIMA HILDA INES</t>
+          <t>MULLO GUACHO ANA LUCIA</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
-        <v>16.74</v>
+        <v>0</v>
       </c>
       <c r="D37" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>1133.57</v>
+        <v>0</v>
       </c>
       <c r="F37" s="2" t="n">
         <v>0</v>
@@ -5277,20 +5097,20 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>MULLO GUACHO ANA LUCIA</t>
+          <t>OCHOA OCAMPO JOHANNA SUSANA</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D38" s="2" t="n">
-        <v>0</v>
+        <v>976.9400000000001</v>
       </c>
       <c r="E38" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>0</v>
+        <v>1052.88</v>
       </c>
       <c r="G38" s="2" t="n">
         <v>0</v>
@@ -5304,23 +5124,23 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>OCHOA OCAMPO JOHANNA SUSANA</t>
+          <t>PAUTA ASTUDILLO JULIO HERNAN</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D39" s="2" t="n">
-        <v>976.9400000000001</v>
+        <v>321.93</v>
       </c>
       <c r="E39" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F39" s="2" t="n">
-        <v>1052.88</v>
+        <v>4867.08</v>
       </c>
       <c r="G39" s="2" t="n">
-        <v>0</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="40">
@@ -5331,23 +5151,23 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>PAUTA ASTUDILLO JULIO HERNAN</t>
+          <t>REYES GUILLEN VICTOR EUGENIO</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
-        <v>0</v>
+        <v>1882.6</v>
       </c>
       <c r="D40" s="2" t="n">
-        <v>321.93</v>
+        <v>0</v>
       </c>
       <c r="E40" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>4867.08</v>
+        <v>4.06</v>
       </c>
       <c r="G40" s="2" t="n">
-        <v>1500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41">
@@ -5358,23 +5178,23 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>QUIÑONEZ LEON MARIA PURIFICACION</t>
+          <t>ROBLES CAMPOVERDE TANIA CRISTINA</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
-        <v>0</v>
+        <v>101.16</v>
       </c>
       <c r="D41" s="2" t="n">
-        <v>0</v>
+        <v>2180.13</v>
       </c>
       <c r="E41" s="2" t="n">
-        <v>0</v>
+        <v>3085.71</v>
       </c>
       <c r="F41" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G41" s="2" t="n">
-        <v>0</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="42">
@@ -5385,11 +5205,11 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>REYES GUILLEN VICTOR EUGENIO</t>
+          <t>ROCAFUERTE LOPEZ EVELYN ESTEFANIA</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
-        <v>1882.6</v>
+        <v>0</v>
       </c>
       <c r="D42" s="2" t="n">
         <v>0</v>
@@ -5398,7 +5218,7 @@
         <v>0</v>
       </c>
       <c r="F42" s="2" t="n">
-        <v>4.06</v>
+        <v>0</v>
       </c>
       <c r="G42" s="2" t="n">
         <v>0</v>
@@ -5412,23 +5232,23 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>ROBLES CAMPOVERDE TANIA CRISTINA</t>
+          <t>RUALES SARAGURO JIMMY JAVIER</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
-        <v>101.16</v>
+        <v>9109.299999999999</v>
       </c>
       <c r="D43" s="2" t="n">
-        <v>2180.13</v>
+        <v>5577.51</v>
       </c>
       <c r="E43" s="2" t="n">
-        <v>3085.71</v>
+        <v>0</v>
       </c>
       <c r="F43" s="2" t="n">
-        <v>0</v>
+        <v>965.67</v>
       </c>
       <c r="G43" s="2" t="n">
-        <v>2000</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="44">
@@ -5439,23 +5259,23 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>ROCAFUERTE LOPEZ EVELYN ESTEFANIA</t>
+          <t>SANDOVAL GONZALEZ NILO GUILLERMO</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D44" s="2" t="n">
-        <v>0</v>
+        <v>1432.86</v>
       </c>
       <c r="E44" s="2" t="n">
-        <v>0</v>
+        <v>-1284.32</v>
       </c>
       <c r="F44" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G44" s="2" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="45">
@@ -5466,23 +5286,23 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>RUALES SARAGURO JIMMY JAVIER</t>
+          <t>SARITAMA HERRERA MARIA ELIZABETH</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
-        <v>9109.299999999999</v>
+        <v>0</v>
       </c>
       <c r="D45" s="2" t="n">
-        <v>5577.51</v>
+        <v>0</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>0</v>
+        <v>474.08</v>
       </c>
       <c r="F45" s="2" t="n">
-        <v>965.67</v>
+        <v>71.11</v>
       </c>
       <c r="G45" s="2" t="n">
-        <v>5000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46">
@@ -5493,23 +5313,23 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>SANDOVAL GONZALEZ NILO GUILLERMO</t>
+          <t>SARMIENTO SARMIENTO SANDRA EULALIA</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D46" s="2" t="n">
-        <v>1432.86</v>
+        <v>0</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>-1284.32</v>
+        <v>0</v>
       </c>
       <c r="F46" s="2" t="n">
-        <v>0</v>
+        <v>1756.19</v>
       </c>
       <c r="G46" s="2" t="n">
-        <v>1200</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="47">
@@ -5520,20 +5340,20 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>SARITAMA HERRERA MARIA ELIZABETH</t>
+          <t>SIMANCAS AGUILAR HONORIO ANTONIO</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
-        <v>0</v>
+        <v>3155.46</v>
       </c>
       <c r="D47" s="2" t="n">
-        <v>0</v>
+        <v>1348.76</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>474.08</v>
+        <v>13692.06</v>
       </c>
       <c r="F47" s="2" t="n">
-        <v>71.11</v>
+        <v>0</v>
       </c>
       <c r="G47" s="2" t="n">
         <v>0</v>
@@ -5547,11 +5367,11 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>SARMIENTO SARMIENTO SANDRA EULALIA</t>
+          <t>TAMAY SANTACRUZ MARIA ANGELICA</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
-        <v>0</v>
+        <v>4237.6</v>
       </c>
       <c r="D48" s="2" t="n">
         <v>0</v>
@@ -5560,10 +5380,10 @@
         <v>0</v>
       </c>
       <c r="F48" s="2" t="n">
-        <v>1756.19</v>
+        <v>37.75</v>
       </c>
       <c r="G48" s="2" t="n">
-        <v>1000</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="49">
@@ -5574,23 +5394,23 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>SIMANCAS AGUILAR HONORIO ANTONIO</t>
+          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
-        <v>3155.46</v>
+        <v>0</v>
       </c>
       <c r="D49" s="2" t="n">
-        <v>1348.76</v>
+        <v>0</v>
       </c>
       <c r="E49" s="2" t="n">
-        <v>13692.06</v>
+        <v>0</v>
       </c>
       <c r="F49" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G49" s="2" t="n">
-        <v>0</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="50">
@@ -5601,7 +5421,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>SOPLIN MENDOZA TABITA</t>
+          <t>VEINTIMILLA JARAMILLO HERMANOS VJHNOS S.A.S.</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
@@ -5628,11 +5448,11 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>TAMAY SANTACRUZ MARIA ANGELICA</t>
+          <t>VERA CABRERA JORGE ENRIQUE</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
-        <v>4237.6</v>
+        <v>0</v>
       </c>
       <c r="D51" s="2" t="n">
         <v>0</v>
@@ -5641,10 +5461,10 @@
         <v>0</v>
       </c>
       <c r="F51" s="2" t="n">
-        <v>37.75</v>
+        <v>0</v>
       </c>
       <c r="G51" s="2" t="n">
-        <v>1500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="52">
@@ -5655,7 +5475,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
+          <t>VIVANCO MALDONADO SILVANA MARILY</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
@@ -5671,104 +5491,23 @@
         <v>0</v>
       </c>
       <c r="G52" s="2" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>VEINTIMILLA JARAMILLO HERMANOS VJHNOS S.A.S.</t>
-        </is>
-      </c>
-      <c r="C53" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D53" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E53" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F53" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G53" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>VERA CABRERA JORGE ENRIQUE</t>
-        </is>
-      </c>
-      <c r="C54" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D54" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E54" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F54" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G54" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>VIVANCO MALDONADO SILVANA MARILY</t>
-        </is>
-      </c>
-      <c r="C55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G55" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="C56" s="4" t="n">
+      <c r="C53" s="4" t="n">
         <v>35603.86</v>
       </c>
-      <c r="D56" s="4" t="n">
+      <c r="D53" s="4" t="n">
         <v>28143.93</v>
       </c>
-      <c r="E56" s="4" t="n">
+      <c r="E53" s="4" t="n">
         <v>43533.43</v>
       </c>
-      <c r="F56" s="4" t="n">
+      <c r="F53" s="4" t="n">
         <v>43936.91</v>
       </c>
-      <c r="G56" s="4" t="n">
+      <c r="G53" s="4" t="n">
         <v>47200</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática 2026-09-29 12:48:34
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R59"/>
+  <dimension ref="A1:R58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1463,7 +1463,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>DIAZ CHAVEZ DIEGO FERNANDO</t>
+          <t>DISTRIBUIDORA VASQUEZ ORDOÑEZ DISTRIVASOR CIA LTDA</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
@@ -1523,7 +1523,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>DISTRIBUIDORA VASQUEZ ORDOÑEZ DISTRIVASOR CIA LTDA</t>
+          <t>ESPINOZA GOMEZ LILIA ROSARIO</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
@@ -1542,16 +1542,16 @@
         <v>0</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>0</v>
+        <v>705.6</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>0</v>
+        <v>297.36</v>
       </c>
       <c r="J18" s="2" t="n">
         <v>0</v>
       </c>
       <c r="K18" s="2" t="n">
-        <v>0</v>
+        <v>1895.04</v>
       </c>
       <c r="L18" s="2" t="n">
         <v>0</v>
@@ -1583,7 +1583,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ESPINOZA GOMEZ LILIA ROSARIO</t>
+          <t>FABIMP BENIGNO BRAVO S.A.S.</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
@@ -1602,22 +1602,22 @@
         <v>0</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>705.6</v>
+        <v>0</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>297.36</v>
+        <v>0</v>
       </c>
       <c r="J19" s="2" t="n">
         <v>0</v>
       </c>
       <c r="K19" s="2" t="n">
-        <v>1895.04</v>
+        <v>0</v>
       </c>
       <c r="L19" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M19" s="2" t="n">
-        <v>0</v>
+        <v>6241.39</v>
       </c>
       <c r="N19" s="2" t="n">
         <v>0</v>
@@ -1643,7 +1643,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>FABIMP BENIGNO BRAVO S.A.S.</t>
+          <t>FERRICENTER EL ARENAL CIA. LTDA.</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
@@ -1677,7 +1677,7 @@
         <v>0</v>
       </c>
       <c r="M20" s="2" t="n">
-        <v>6241.39</v>
+        <v>0</v>
       </c>
       <c r="N20" s="2" t="n">
         <v>0</v>
@@ -1703,7 +1703,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>FERRICENTER EL ARENAL CIA. LTDA.</t>
+          <t>FERRICRAFT S.A.S.</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
@@ -1763,7 +1763,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>FERRICRAFT S.A.S.</t>
+          <t>FRANK FERRETERIA FRANKFERRE CIA.</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
@@ -1823,7 +1823,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>FRANK FERRETERIA FRANKFERRE CIA.</t>
+          <t>GLOBAL MOYANO &amp; ASOCIADOS LEMO S.A.S.</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
@@ -1857,7 +1857,7 @@
         <v>0</v>
       </c>
       <c r="M23" s="2" t="n">
-        <v>0</v>
+        <v>6.32</v>
       </c>
       <c r="N23" s="2" t="n">
         <v>0</v>
@@ -1883,7 +1883,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>GLOBAL MOYANO &amp; ASOCIADOS LEMO S.A.S.</t>
+          <t>GRANDA SANDOVAL JACKELINE ELIZABETH</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
@@ -1917,7 +1917,7 @@
         <v>0</v>
       </c>
       <c r="M24" s="2" t="n">
-        <v>6.32</v>
+        <v>0</v>
       </c>
       <c r="N24" s="2" t="n">
         <v>0</v>
@@ -1943,7 +1943,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>GRANDA SANDOVAL JACKELINE ELIZABETH</t>
+          <t>HUERTA MUÑOZ NANCY ELIZABETH</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
@@ -2003,7 +2003,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>HUERTA MUÑOZ NANCY ELIZABETH</t>
+          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
@@ -2013,7 +2013,7 @@
         <v>0</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>0</v>
+        <v>65.79000000000001</v>
       </c>
       <c r="F26" s="2" t="n">
         <v>0</v>
@@ -2063,7 +2063,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
+          <t>IMPORTADORA ORTEGA CIA. LTDA.</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
@@ -2073,7 +2073,7 @@
         <v>0</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>65.79000000000001</v>
+        <v>0</v>
       </c>
       <c r="F27" s="2" t="n">
         <v>0</v>
@@ -2085,7 +2085,7 @@
         <v>0</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>0</v>
+        <v>1830.72</v>
       </c>
       <c r="J27" s="2" t="n">
         <v>0</v>
@@ -2097,7 +2097,7 @@
         <v>0</v>
       </c>
       <c r="M27" s="2" t="n">
-        <v>0</v>
+        <v>5779.47</v>
       </c>
       <c r="N27" s="2" t="n">
         <v>0</v>
@@ -2123,17 +2123,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>IMPORTADORA ORTEGA CIA. LTDA.</t>
+          <t>JIMBO BRITO SELENE PATRICIA</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>0</v>
+        <v>436.55</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>0</v>
+        <v>417.01</v>
       </c>
       <c r="F28" s="2" t="n">
         <v>0</v>
@@ -2142,22 +2142,22 @@
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>0</v>
+        <v>247.5</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>1830.72</v>
+        <v>350.77</v>
       </c>
       <c r="J28" s="2" t="n">
         <v>0</v>
       </c>
       <c r="K28" s="2" t="n">
-        <v>0</v>
+        <v>363.16</v>
       </c>
       <c r="L28" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M28" s="2" t="n">
-        <v>5779.47</v>
+        <v>1918.73</v>
       </c>
       <c r="N28" s="2" t="n">
         <v>0</v>
@@ -2183,17 +2183,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>JIMBO BRITO SELENE PATRICIA</t>
+          <t>JIMENEZ GORDILLO LADY KARINA</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>436.55</v>
+        <v>0</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>417.01</v>
+        <v>0</v>
       </c>
       <c r="F29" s="2" t="n">
         <v>0</v>
@@ -2202,22 +2202,22 @@
         <v>0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>247.5</v>
+        <v>0</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>350.77</v>
+        <v>0</v>
       </c>
       <c r="J29" s="2" t="n">
         <v>0</v>
       </c>
       <c r="K29" s="2" t="n">
-        <v>363.16</v>
+        <v>0</v>
       </c>
       <c r="L29" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M29" s="2" t="n">
-        <v>1918.73</v>
+        <v>0</v>
       </c>
       <c r="N29" s="2" t="n">
         <v>0</v>
@@ -2243,7 +2243,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>JIMENEZ GORDILLO LADY KARINA</t>
+          <t>JUAREZ FLORES JORGE WILLIAMS</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
@@ -2303,7 +2303,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>JUAREZ FLORES JORGE WILLIAMS</t>
+          <t>LEMA ESPINOZA MANUEL MARIA</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
@@ -2363,7 +2363,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>LEMA ESPINOZA MANUEL MARIA</t>
+          <t>MARIN SANCHEZ GABRIEL ALEXANDER</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
@@ -2385,13 +2385,13 @@
         <v>0</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>0</v>
+        <v>184.95</v>
       </c>
       <c r="J32" s="2" t="n">
         <v>0</v>
       </c>
       <c r="K32" s="2" t="n">
-        <v>0</v>
+        <v>201.32</v>
       </c>
       <c r="L32" s="2" t="n">
         <v>0</v>
@@ -2423,7 +2423,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>MARIN SANCHEZ GABRIEL ALEXANDER</t>
+          <t>MEGGA-FRANK SAS</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
@@ -2442,22 +2442,22 @@
         <v>0</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>0</v>
+        <v>615.6</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>184.95</v>
+        <v>551.99</v>
       </c>
       <c r="J33" s="2" t="n">
         <v>0</v>
       </c>
       <c r="K33" s="2" t="n">
-        <v>201.32</v>
+        <v>0</v>
       </c>
       <c r="L33" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M33" s="2" t="n">
-        <v>0</v>
+        <v>5710.6</v>
       </c>
       <c r="N33" s="2" t="n">
         <v>0</v>
@@ -2483,7 +2483,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>MEGGA-FRANK SAS</t>
+          <t>MENESES TORRES OSCAR LEONARDO</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
@@ -2502,10 +2502,10 @@
         <v>0</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>615.6</v>
+        <v>0</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>551.99</v>
+        <v>0</v>
       </c>
       <c r="J34" s="2" t="n">
         <v>0</v>
@@ -2517,7 +2517,7 @@
         <v>0</v>
       </c>
       <c r="M34" s="2" t="n">
-        <v>5710.6</v>
+        <v>0</v>
       </c>
       <c r="N34" s="2" t="n">
         <v>0</v>
@@ -2543,7 +2543,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>MENESES TORRES OSCAR LEONARDO</t>
+          <t>MIM CONSTRUFERRETERIA E IMPORTADORA SAS</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
@@ -2603,7 +2603,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>MIM CONSTRUFERRETERIA E IMPORTADORA SAS</t>
+          <t>MONTAÑO JIMENEZ SANDRA GABRIELA</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
@@ -2663,7 +2663,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>MONTAÑO JIMENEZ SANDRA GABRIELA</t>
+          <t>MORALES GRACIELA ENITH</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
@@ -2723,7 +2723,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>MORALES GRACIELA ENITH</t>
+          <t>MOROCHO BACUILIMA HILDA INES</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>MOROCHO BACUILIMA HILDA INES</t>
+          <t>MULLO GUACHO ANA LUCIA</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
@@ -2843,7 +2843,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>MULLO GUACHO ANA LUCIA</t>
+          <t>OCHOA OCAMPO JOHANNA SUSANA</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
@@ -2871,7 +2871,7 @@
         <v>0</v>
       </c>
       <c r="K40" s="2" t="n">
-        <v>0</v>
+        <v>367.08</v>
       </c>
       <c r="L40" s="2" t="n">
         <v>0</v>
@@ -2880,7 +2880,7 @@
         <v>0</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>0</v>
+        <v>685.8</v>
       </c>
       <c r="O40" s="2" t="n">
         <v>0</v>
@@ -2903,7 +2903,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>OCHOA OCAMPO JOHANNA SUSANA</t>
+          <t>ORTIZ GRANDA ANDREA DEL CISNE</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
@@ -2931,7 +2931,7 @@
         <v>0</v>
       </c>
       <c r="K41" s="2" t="n">
-        <v>367.08</v>
+        <v>0</v>
       </c>
       <c r="L41" s="2" t="n">
         <v>0</v>
@@ -2940,7 +2940,7 @@
         <v>0</v>
       </c>
       <c r="N41" s="2" t="n">
-        <v>685.8</v>
+        <v>0</v>
       </c>
       <c r="O41" s="2" t="n">
         <v>0</v>
@@ -2963,7 +2963,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>ORTIZ GRANDA ANDREA DEL CISNE</t>
+          <t>PAUTA ASTUDILLO JULIO HERNAN</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
@@ -2997,7 +2997,7 @@
         <v>0</v>
       </c>
       <c r="M42" s="2" t="n">
-        <v>0</v>
+        <v>4835</v>
       </c>
       <c r="N42" s="2" t="n">
         <v>0</v>
@@ -3023,7 +3023,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>PAUTA ASTUDILLO JULIO HERNAN</t>
+          <t>REYES GUILLEN VICTOR EUGENIO</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
@@ -3057,7 +3057,7 @@
         <v>0</v>
       </c>
       <c r="M43" s="2" t="n">
-        <v>4835</v>
+        <v>0</v>
       </c>
       <c r="N43" s="2" t="n">
         <v>0</v>
@@ -3083,7 +3083,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>REYES GUILLEN VICTOR EUGENIO</t>
+          <t>ROBLES CAMPOVERDE TANIA CRISTINA</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
@@ -3143,7 +3143,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>ROBLES CAMPOVERDE TANIA CRISTINA</t>
+          <t>ROCAFUERTE LOPEZ EVELYN ESTEFANIA</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
@@ -3203,7 +3203,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>ROCAFUERTE LOPEZ EVELYN ESTEFANIA</t>
+          <t>RUALES SARAGURO JIMMY JAVIER</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
@@ -3237,7 +3237,7 @@
         <v>0</v>
       </c>
       <c r="M46" s="2" t="n">
-        <v>0</v>
+        <v>926.02</v>
       </c>
       <c r="N46" s="2" t="n">
         <v>0</v>
@@ -3263,7 +3263,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>RUALES SARAGURO JIMMY JAVIER</t>
+          <t>SANDOVAL GONZALEZ LAUTARO MARCELO</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
@@ -3297,7 +3297,7 @@
         <v>0</v>
       </c>
       <c r="M47" s="2" t="n">
-        <v>926.02</v>
+        <v>0</v>
       </c>
       <c r="N47" s="2" t="n">
         <v>0</v>
@@ -3323,7 +3323,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>SANDOVAL GONZALEZ LAUTARO MARCELO</t>
+          <t>SANDOVAL GONZALEZ NILO GUILLERMO</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
@@ -3383,7 +3383,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>SANDOVAL GONZALEZ NILO GUILLERMO</t>
+          <t>SANDOVAL MONTAÑO MARICELA DEL CISNE</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
@@ -3443,7 +3443,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>SANDOVAL MONTAÑO MARICELA DEL CISNE</t>
+          <t>SARITAMA HERRERA MARIA ELIZABETH</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
@@ -3477,7 +3477,7 @@
         <v>0</v>
       </c>
       <c r="M50" s="2" t="n">
-        <v>0</v>
+        <v>71.11</v>
       </c>
       <c r="N50" s="2" t="n">
         <v>0</v>
@@ -3503,7 +3503,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>SARITAMA HERRERA MARIA ELIZABETH</t>
+          <t>SARMIENTO SARMIENTO SANDRA EULALIA</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
@@ -3513,7 +3513,7 @@
         <v>0</v>
       </c>
       <c r="E51" s="2" t="n">
-        <v>0</v>
+        <v>205.95</v>
       </c>
       <c r="F51" s="2" t="n">
         <v>0</v>
@@ -3537,7 +3537,7 @@
         <v>0</v>
       </c>
       <c r="M51" s="2" t="n">
-        <v>71.11</v>
+        <v>1550.24</v>
       </c>
       <c r="N51" s="2" t="n">
         <v>0</v>
@@ -3563,7 +3563,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>SARMIENTO SARMIENTO SANDRA EULALIA</t>
+          <t>SIMANCAS AGUILAR HONORIO ANTONIO</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
@@ -3573,7 +3573,7 @@
         <v>0</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>205.95</v>
+        <v>0</v>
       </c>
       <c r="F52" s="2" t="n">
         <v>0</v>
@@ -3597,7 +3597,7 @@
         <v>0</v>
       </c>
       <c r="M52" s="2" t="n">
-        <v>1550.24</v>
+        <v>0</v>
       </c>
       <c r="N52" s="2" t="n">
         <v>0</v>
@@ -3623,7 +3623,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>SIMANCAS AGUILAR HONORIO ANTONIO</t>
+          <t>TAMAY SANTACRUZ MARIA ANGELICA</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
@@ -3683,7 +3683,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>TAMAY SANTACRUZ MARIA ANGELICA</t>
+          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
@@ -3743,7 +3743,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>VALENCIA RUIZ FAUSTO GABRIEL</t>
+          <t>VEINTIMILLA JARAMILLO HERMANOS VJHNOS S.A.S.</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
@@ -3803,7 +3803,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>VEINTIMILLA JARAMILLO HERMANOS VJHNOS S.A.S.</t>
+          <t>VERA CABRERA JORGE ENRIQUE</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
@@ -3863,7 +3863,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>VERA CABRERA JORGE ENRIQUE</t>
+          <t>VIVANCO MALDONADO SILVANA MARILY</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
@@ -3916,144 +3916,84 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>ILLER LOPEZ ROBERTO FERNANDO</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>VIVANCO MALDONADO SILVANA MARILY</t>
-        </is>
-      </c>
-      <c r="C58" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D58" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E58" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F58" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G58" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H58" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I58" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J58" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K58" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L58" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M58" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N58" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O58" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P58" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q58" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R58" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="C59" s="3" t="inlineStr">
-        <is>
-          <t>0 de 57</t>
-        </is>
-      </c>
-      <c r="D59" s="3" t="inlineStr">
-        <is>
-          <t>1 de 57</t>
-        </is>
-      </c>
-      <c r="E59" s="3" t="inlineStr">
-        <is>
-          <t>4 de 57</t>
-        </is>
-      </c>
-      <c r="F59" s="3" t="inlineStr">
-        <is>
-          <t>0 de 57</t>
-        </is>
-      </c>
-      <c r="G59" s="3" t="inlineStr">
-        <is>
-          <t>0 de 57</t>
-        </is>
-      </c>
-      <c r="H59" s="3" t="inlineStr">
-        <is>
-          <t>6 de 57</t>
-        </is>
-      </c>
-      <c r="I59" s="3" t="inlineStr">
-        <is>
-          <t>7 de 57</t>
-        </is>
-      </c>
-      <c r="J59" s="3" t="inlineStr">
-        <is>
-          <t>0 de 57</t>
-        </is>
-      </c>
-      <c r="K59" s="3" t="inlineStr">
-        <is>
-          <t>5 de 57</t>
-        </is>
-      </c>
-      <c r="L59" s="3" t="inlineStr">
-        <is>
-          <t>1 de 57</t>
-        </is>
-      </c>
-      <c r="M59" s="3" t="inlineStr">
-        <is>
-          <t>13 de 57</t>
-        </is>
-      </c>
-      <c r="N59" s="3" t="inlineStr">
-        <is>
-          <t>1 de 57</t>
-        </is>
-      </c>
-      <c r="O59" s="3" t="inlineStr">
-        <is>
-          <t>0 de 57</t>
-        </is>
-      </c>
-      <c r="P59" s="3" t="inlineStr">
-        <is>
-          <t>0 de 57</t>
-        </is>
-      </c>
-      <c r="Q59" s="3" t="inlineStr">
-        <is>
-          <t>0 de 57</t>
-        </is>
-      </c>
-      <c r="R59" s="3" t="inlineStr">
-        <is>
-          <t>0 de 57</t>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>0 de 56</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>1 de 56</t>
+        </is>
+      </c>
+      <c r="E58" s="3" t="inlineStr">
+        <is>
+          <t>4 de 56</t>
+        </is>
+      </c>
+      <c r="F58" s="3" t="inlineStr">
+        <is>
+          <t>0 de 56</t>
+        </is>
+      </c>
+      <c r="G58" s="3" t="inlineStr">
+        <is>
+          <t>0 de 56</t>
+        </is>
+      </c>
+      <c r="H58" s="3" t="inlineStr">
+        <is>
+          <t>6 de 56</t>
+        </is>
+      </c>
+      <c r="I58" s="3" t="inlineStr">
+        <is>
+          <t>7 de 56</t>
+        </is>
+      </c>
+      <c r="J58" s="3" t="inlineStr">
+        <is>
+          <t>0 de 56</t>
+        </is>
+      </c>
+      <c r="K58" s="3" t="inlineStr">
+        <is>
+          <t>5 de 56</t>
+        </is>
+      </c>
+      <c r="L58" s="3" t="inlineStr">
+        <is>
+          <t>1 de 56</t>
+        </is>
+      </c>
+      <c r="M58" s="3" t="inlineStr">
+        <is>
+          <t>13 de 56</t>
+        </is>
+      </c>
+      <c r="N58" s="3" t="inlineStr">
+        <is>
+          <t>1 de 56</t>
+        </is>
+      </c>
+      <c r="O58" s="3" t="inlineStr">
+        <is>
+          <t>0 de 56</t>
+        </is>
+      </c>
+      <c r="P58" s="3" t="inlineStr">
+        <is>
+          <t>0 de 56</t>
+        </is>
+      </c>
+      <c r="Q58" s="3" t="inlineStr">
+        <is>
+          <t>0 de 56</t>
+        </is>
+      </c>
+      <c r="R58" s="3" t="inlineStr">
+        <is>
+          <t>0 de 56</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática 2026-09-30 13:30:18
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -573,16 +573,16 @@
         <v>0</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>0</v>
+        <v>148.72</v>
       </c>
       <c r="F2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>0</v>
+        <v>169.89</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>0</v>
+        <v>782.1</v>
       </c>
       <c r="I2" s="2" t="n">
         <v>0</v>
@@ -597,7 +597,7 @@
         <v>0</v>
       </c>
       <c r="M2" s="2" t="n">
-        <v>0</v>
+        <v>2758.28</v>
       </c>
       <c r="N2" s="2" t="n">
         <v>0</v>
@@ -1365,7 +1365,7 @@
         <v>0</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>0</v>
+        <v>75.27</v>
       </c>
       <c r="J15" s="2" t="n">
         <v>0</v>
@@ -1377,7 +1377,7 @@
         <v>0</v>
       </c>
       <c r="M15" s="2" t="n">
-        <v>0</v>
+        <v>1950.44</v>
       </c>
       <c r="N15" s="2" t="n">
         <v>0</v>
@@ -2130,7 +2130,7 @@
         <v>0</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>436.55</v>
+        <v>706.3</v>
       </c>
       <c r="E28" s="2" t="n">
         <v>417.01</v>
@@ -2142,7 +2142,7 @@
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>247.5</v>
+        <v>318.6</v>
       </c>
       <c r="I28" s="2" t="n">
         <v>350.77</v>
@@ -2151,13 +2151,13 @@
         <v>0</v>
       </c>
       <c r="K28" s="2" t="n">
-        <v>363.16</v>
+        <v>406.56</v>
       </c>
       <c r="L28" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M28" s="2" t="n">
-        <v>1918.73</v>
+        <v>2078.91</v>
       </c>
       <c r="N28" s="2" t="n">
         <v>0</v>
@@ -2880,7 +2880,7 @@
         <v>0</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>685.8</v>
+        <v>1371.6</v>
       </c>
       <c r="O40" s="2" t="n">
         <v>0</v>
@@ -3117,7 +3117,7 @@
         <v>0</v>
       </c>
       <c r="M44" s="2" t="n">
-        <v>0</v>
+        <v>1623.88</v>
       </c>
       <c r="N44" s="2" t="n">
         <v>0</v>
@@ -3928,7 +3928,7 @@
       </c>
       <c r="E58" s="3" t="inlineStr">
         <is>
-          <t>4 de 56</t>
+          <t>5 de 56</t>
         </is>
       </c>
       <c r="F58" s="3" t="inlineStr">
@@ -3938,24 +3938,24 @@
       </c>
       <c r="G58" s="3" t="inlineStr">
         <is>
+          <t>1 de 56</t>
+        </is>
+      </c>
+      <c r="H58" s="3" t="inlineStr">
+        <is>
+          <t>7 de 56</t>
+        </is>
+      </c>
+      <c r="I58" s="3" t="inlineStr">
+        <is>
+          <t>8 de 56</t>
+        </is>
+      </c>
+      <c r="J58" s="3" t="inlineStr">
+        <is>
           <t>0 de 56</t>
         </is>
       </c>
-      <c r="H58" s="3" t="inlineStr">
-        <is>
-          <t>6 de 56</t>
-        </is>
-      </c>
-      <c r="I58" s="3" t="inlineStr">
-        <is>
-          <t>7 de 56</t>
-        </is>
-      </c>
-      <c r="J58" s="3" t="inlineStr">
-        <is>
-          <t>0 de 56</t>
-        </is>
-      </c>
       <c r="K58" s="3" t="inlineStr">
         <is>
           <t>5 de 56</t>
@@ -3968,7 +3968,7 @@
       </c>
       <c r="M58" s="3" t="inlineStr">
         <is>
-          <t>13 de 56</t>
+          <t>16 de 56</t>
         </is>
       </c>
       <c r="N58" s="3" t="inlineStr">
@@ -4105,7 +4105,7 @@
         <v>0</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>10.15</v>
+        <v>3869.14</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>2000</v>
@@ -4456,7 +4456,7 @@
         <v>5446.06</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>0</v>
+        <v>2025.71</v>
       </c>
       <c r="G16" s="2" t="n">
         <v>1500</v>
@@ -4753,7 +4753,7 @@
         <v>0</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>5097.28</v>
+        <v>6901.37</v>
       </c>
       <c r="G27" s="2" t="n">
         <v>0</v>
@@ -5050,7 +5050,7 @@
         <v>0</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>1052.88</v>
+        <v>1738.68</v>
       </c>
       <c r="G38" s="2" t="n">
         <v>0</v>
@@ -5131,7 +5131,7 @@
         <v>3085.71</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>0</v>
+        <v>1623.88</v>
       </c>
       <c r="G41" s="2" t="n">
         <v>2000</v>
@@ -5445,7 +5445,7 @@
         <v>43533.43</v>
       </c>
       <c r="F53" s="4" t="n">
-        <v>43904.83</v>
+        <v>53903.3</v>
       </c>
       <c r="G53" s="4" t="n">
         <v>47200</v>
@@ -5469,8 +5469,8 @@
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5520,13 +5520,13 @@
         <v>2600</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>436.55</v>
+        <v>706.3</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>2163.45</v>
+        <v>1893.7</v>
       </c>
       <c r="F2" s="5" t="n">
-        <v>0.1679038461538462</v>
+        <v>0.2716538461538461</v>
       </c>
     </row>
     <row r="3">
@@ -5544,13 +5544,13 @@
         <v>4001</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>108.9</v>
+        <v>1368.56</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>3892.1</v>
+        <v>2632.44</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>0.02721819545113722</v>
+        <v>0.3420544863784054</v>
       </c>
     </row>
     <row r="4">
@@ -5568,13 +5568,13 @@
         <v>199.5</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>886.13</v>
+        <v>1034.85</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>-686.63</v>
+        <v>-835.3499999999999</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>4.441754385964912</v>
+        <v>5.187218045112782</v>
       </c>
     </row>
     <row r="5">
@@ -5592,13 +5592,13 @@
         <v>198.5</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0</v>
+        <v>169.89</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>198.5</v>
+        <v>28.61000000000001</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0</v>
+        <v>0.8558690176322418</v>
       </c>
     </row>
     <row r="6">
@@ -5616,13 +5616,13 @@
         <v>697</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>2827.53</v>
+        <v>3680.73</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>-2130.53</v>
+        <v>-2983.73</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>4.056714490674318</v>
+        <v>5.280817790530847</v>
       </c>
     </row>
     <row r="7">
@@ -5640,13 +5640,13 @@
         <v>463</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>3689.65</v>
+        <v>3764.92</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>-3226.65</v>
+        <v>-3301.92</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>7.969006479481641</v>
+        <v>8.131576673866091</v>
       </c>
     </row>
     <row r="8">
@@ -5664,10 +5664,10 @@
         <v>0</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>685.8</v>
+        <v>1371.6</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>-685.8</v>
+        <v>-1371.6</v>
       </c>
       <c r="F8" s="5" t="n">
         <v>0</v>
@@ -5688,13 +5688,13 @@
         <v>203.76</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>3039.78</v>
+        <v>3083.18</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>-2836.02</v>
+        <v>-2879.42</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>14.91843345111896</v>
+        <v>15.13142913231252</v>
       </c>
     </row>
     <row r="10">
@@ -5760,13 +5760,13 @@
         <v>39603</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>29815.96</v>
+        <v>36308.74</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>9787.040000000001</v>
+        <v>3294.260000000002</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0.7528712471277428</v>
+        <v>0.9168179178345074</v>
       </c>
     </row>
     <row r="13">
@@ -5779,13 +5779,13 @@
         <v>49040.76</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>43970.62</v>
+        <v>53969.09</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>5070.139999999999</v>
+        <v>-4928.329999999998</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>0.8966137555780129</v>
+        <v>1.100494568191847</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-15 15:30:17
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -2931,7 +2931,7 @@
         <v>0</v>
       </c>
       <c r="K41" s="2" t="n">
-        <v>0</v>
+        <v>236.88</v>
       </c>
       <c r="L41" s="2" t="n">
         <v>0</v>
@@ -2940,7 +2940,7 @@
         <v>0</v>
       </c>
       <c r="N41" s="2" t="n">
-        <v>0</v>
+        <v>685.8</v>
       </c>
       <c r="O41" s="2" t="n">
         <v>0</v>
@@ -4018,14 +4018,14 @@
       </c>
       <c r="K59" s="3" t="inlineStr">
         <is>
+          <t>1 de 57</t>
+        </is>
+      </c>
+      <c r="L59" s="3" t="inlineStr">
+        <is>
           <t>0 de 57</t>
         </is>
       </c>
-      <c r="L59" s="3" t="inlineStr">
-        <is>
-          <t>0 de 57</t>
-        </is>
-      </c>
       <c r="M59" s="3" t="inlineStr">
         <is>
           <t>4 de 57</t>
@@ -4033,7 +4033,7 @@
       </c>
       <c r="N59" s="3" t="inlineStr">
         <is>
-          <t>0 de 57</t>
+          <t>1 de 57</t>
         </is>
       </c>
       <c r="O59" s="3" t="inlineStr">
@@ -5164,7 +5164,7 @@
         <v>1738.68</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>0</v>
+        <v>1038.68</v>
       </c>
       <c r="G40" s="2" t="n">
         <v>0</v>
@@ -5559,7 +5559,7 @@
         <v>53903.3</v>
       </c>
       <c r="F55" s="4" t="n">
-        <v>1597.71</v>
+        <v>2636.39</v>
       </c>
       <c r="G55" s="4" t="n">
         <v>32500</v>
@@ -5778,10 +5778,10 @@
         <v>0</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>0</v>
+        <v>685.8</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>0</v>
+        <v>-685.8</v>
       </c>
       <c r="F8" s="5" t="n">
         <v>0</v>
@@ -5802,13 +5802,13 @@
         <v>203.76</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0</v>
+        <v>236.88</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>203.76</v>
+        <v>-33.12</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>0</v>
+        <v>1.162544169611307</v>
       </c>
     </row>
     <row r="10">
@@ -5826,13 +5826,13 @@
         <v>115</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>116</v>
+        <v>232</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>-1</v>
+        <v>-117</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>1.008695652173913</v>
+        <v>2.017391304347826</v>
       </c>
     </row>
     <row r="11">
@@ -5893,13 +5893,13 @@
         <v>49194.01</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>1597.71</v>
+        <v>2636.39</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>47596.3</v>
+        <v>46557.62</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>0.03247773458597907</v>
+        <v>0.05359168728062624</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-20 11:30:16
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -3897,7 +3897,7 @@
         <v>0</v>
       </c>
       <c r="M57" s="2" t="n">
-        <v>0</v>
+        <v>4215.96</v>
       </c>
       <c r="N57" s="2" t="n">
         <v>0</v>
@@ -4028,7 +4028,7 @@
       </c>
       <c r="M59" s="3" t="inlineStr">
         <is>
-          <t>6 de 57</t>
+          <t>7 de 57</t>
         </is>
       </c>
       <c r="N59" s="3" t="inlineStr">
@@ -5515,7 +5515,7 @@
         <v>0</v>
       </c>
       <c r="F53" s="2" t="n">
-        <v>0</v>
+        <v>4215.96</v>
       </c>
       <c r="G53" s="2" t="n">
         <v>0</v>
@@ -5559,7 +5559,7 @@
         <v>53903.3</v>
       </c>
       <c r="F55" s="4" t="n">
-        <v>11627.49</v>
+        <v>15843.45</v>
       </c>
       <c r="G55" s="4" t="n">
         <v>32500</v>
@@ -5582,7 +5582,7 @@
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
     <col width="25" customWidth="1" min="6" max="6"/>
   </cols>
@@ -5874,13 +5874,13 @@
         <v>40601.25</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>9766.33</v>
+        <v>13982.29</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>30834.92</v>
+        <v>26618.96</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0.2405425941319541</v>
+        <v>0.344380776453927</v>
       </c>
     </row>
     <row r="13">
@@ -5893,13 +5893,13 @@
         <v>49194.01</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>11627.49</v>
+        <v>15843.45</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>37566.52</v>
+        <v>33350.56</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>0.2363598738952161</v>
+        <v>0.3220605516809872</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-21 15:30:17
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -891,7 +891,7 @@
         <v>0</v>
       </c>
       <c r="K7" s="2" t="n">
-        <v>0</v>
+        <v>248.72</v>
       </c>
       <c r="L7" s="2" t="n">
         <v>0</v>
@@ -4018,7 +4018,7 @@
       </c>
       <c r="K59" s="3" t="inlineStr">
         <is>
-          <t>1 de 57</t>
+          <t>2 de 57</t>
         </is>
       </c>
       <c r="L59" s="3" t="inlineStr">
@@ -4327,7 +4327,7 @@
         <v>708.88</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>0</v>
+        <v>259.6</v>
       </c>
       <c r="G9" s="2" t="n">
         <v>1000</v>
@@ -5559,7 +5559,7 @@
         <v>53903.3</v>
       </c>
       <c r="F55" s="4" t="n">
-        <v>15891.35</v>
+        <v>16150.95</v>
       </c>
       <c r="G55" s="4" t="n">
         <v>32500</v>
@@ -5658,13 +5658,13 @@
         <v>4001</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>781.75</v>
+        <v>792.63</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>3219.25</v>
+        <v>3208.37</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>0.1953886528367908</v>
+        <v>0.1981079730067483</v>
       </c>
     </row>
     <row r="4">
@@ -5802,13 +5802,13 @@
         <v>203.76</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>236.88</v>
+        <v>485.6</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>-33.12</v>
+        <v>-281.84</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>1.162544169611307</v>
+        <v>2.383195916764822</v>
       </c>
     </row>
     <row r="10">
@@ -5893,13 +5893,13 @@
         <v>49194.01</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>15891.35</v>
+        <v>16150.95</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>33302.66</v>
+        <v>33043.06</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>0.3230342474622419</v>
+        <v>0.3283113126984363</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-29 16:30:18
</commit_message>
<xml_diff>
--- a/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
+++ b/data/ILLER LOPEZ ROBERTO FERNANDO.xlsx
@@ -2517,7 +2517,7 @@
         <v>0</v>
       </c>
       <c r="M34" s="2" t="n">
-        <v>4846.2</v>
+        <v>4852.1</v>
       </c>
       <c r="N34" s="2" t="n">
         <v>0</v>
@@ -3171,7 +3171,7 @@
         <v>0</v>
       </c>
       <c r="K45" s="2" t="n">
-        <v>0</v>
+        <v>17.91</v>
       </c>
       <c r="L45" s="2" t="n">
         <v>0</v>
@@ -3297,7 +3297,7 @@
         <v>0</v>
       </c>
       <c r="M47" s="2" t="n">
-        <v>7263.33</v>
+        <v>11808.11</v>
       </c>
       <c r="N47" s="2" t="n">
         <v>0</v>
@@ -4018,7 +4018,7 @@
       </c>
       <c r="K59" s="3" t="inlineStr">
         <is>
-          <t>3 de 57</t>
+          <t>4 de 57</t>
         </is>
       </c>
       <c r="L59" s="3" t="inlineStr">
@@ -4076,7 +4076,7 @@
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -5002,7 +5002,7 @@
         <v>6878.19</v>
       </c>
       <c r="F34" s="2" t="n">
-        <v>4846.2</v>
+        <v>4852.1</v>
       </c>
       <c r="G34" s="2" t="n">
         <v>2000</v>
@@ -5245,7 +5245,7 @@
         <v>1623.88</v>
       </c>
       <c r="F43" s="2" t="n">
-        <v>0</v>
+        <v>17.91</v>
       </c>
       <c r="G43" s="2" t="n">
         <v>0</v>
@@ -5299,7 +5299,7 @@
         <v>965.67</v>
       </c>
       <c r="F45" s="2" t="n">
-        <v>7274.45</v>
+        <v>11819.23</v>
       </c>
       <c r="G45" s="2" t="n">
         <v>10000</v>
@@ -5559,7 +5559,7 @@
         <v>53903.3</v>
       </c>
       <c r="F55" s="4" t="n">
-        <v>29031.58</v>
+        <v>33600.17</v>
       </c>
       <c r="G55" s="4" t="n">
         <v>32500</v>
@@ -5802,13 +5802,13 @@
         <v>203.76</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>1361.96</v>
+        <v>1379.87</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>-1158.2</v>
+        <v>-1176.11</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>6.684138201806046</v>
+        <v>6.772035728307813</v>
       </c>
     </row>
     <row r="10">
@@ -5874,13 +5874,13 @@
         <v>40601.25</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>26251.64</v>
+        <v>30802.32</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>14349.61</v>
+        <v>9798.93</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0.6465722114466919</v>
+        <v>0.7586544749238016</v>
       </c>
     </row>
     <row r="13">
@@ -5893,13 +5893,13 @@
         <v>49194.01</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>29031.58</v>
+        <v>33600.17</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>20162.43</v>
+        <v>15593.84</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>0.5901446131348105</v>
+        <v>0.683013440050933</v>
       </c>
     </row>
   </sheetData>

</xml_diff>